<commit_message>
25 de octubre de 2021 v1
</commit_message>
<xml_diff>
--- a/_downloads/0fadcc9aeba798b6b08d9143e4476fd3/Ejemplos distribuciones de probabilidad.xlsx
+++ b/_downloads/0fadcc9aeba798b6b08d9143e4476fd3/Ejemplos distribuciones de probabilidad.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\migue\Dropbox\ITM\ANÁLISIS DE RIESGOS\Archivos de Excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{304F6225-88F7-4C70-9332-13372A315B5C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E7E35808-6EB2-42B6-8ED9-B6A828BC449C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" activeTab="2" xr2:uid="{C33B7364-5EEF-46A0-A185-DDCEC781240D}"/>
   </bookViews>
@@ -408,9 +408,6 @@
     <t>&gt;=SI(B50&lt;=C45;(B50-C44)^2/((C45-C44)*(C46-C44));1-(C46-B50)^2/((C46-C45)*(C46-C44)))</t>
   </si>
   <si>
-    <t>&gt;=SI(A53&lt;=(C45-C44)/(C46-C44);C44+RAIZ(A53*C45*(C46-C44));C46+RAIZ((1-A53)*(C45-C44)*(C46-C44)))</t>
-  </si>
-  <si>
     <t>&gt;=1/(B64-B63)</t>
   </si>
   <si>
@@ -428,6 +425,9 @@
   <si>
     <t>&gt;=DISTR.LOG.INV(A98;C82;C83)</t>
   </si>
+  <si>
+    <t>&gt;=SI(A53&lt;=(C45-C44)/(C46-C44);C44+RAIZ(A53*(C45-C44)*(C46-C44));C46-RAIZ((1-A53)*(C45-C44)*(C46-C44)))</t>
+  </si>
 </sst>
 </file>
 
@@ -439,9 +439,9 @@
     <numFmt numFmtId="165" formatCode="0.0%"/>
     <numFmt numFmtId="166" formatCode="0.000%"/>
     <numFmt numFmtId="167" formatCode="0.0000%"/>
-    <numFmt numFmtId="169" formatCode="0.000000%"/>
-    <numFmt numFmtId="170" formatCode="0.0000000%"/>
-    <numFmt numFmtId="173" formatCode="0.00000"/>
+    <numFmt numFmtId="168" formatCode="0.000000%"/>
+    <numFmt numFmtId="169" formatCode="0.0000000%"/>
+    <numFmt numFmtId="170" formatCode="0.00000"/>
   </numFmts>
   <fonts count="5" x14ac:knownFonts="1">
     <font>
@@ -601,28 +601,19 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="173" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="170" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="165" fontId="3" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="169" fontId="3" fillId="2" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="168" fontId="3" fillId="2" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="165" fontId="3" fillId="2" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="170" fontId="3" fillId="2" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="169" fontId="3" fillId="2" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="6" fontId="3" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
@@ -630,6 +621,15 @@
     </xf>
     <xf numFmtId="2" fontId="3" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -2830,8 +2830,8 @@
       <xdr:row>33</xdr:row>
       <xdr:rowOff>165734</xdr:rowOff>
     </xdr:to>
-    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-      <mc:Choice xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" Requires="a14">
+    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+      <mc:Choice Requires="a14">
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
             <xdr:cNvPr id="2" name="CuadroTexto 6">
@@ -3019,7 +3019,7 @@
           </xdr:txBody>
         </xdr:sp>
       </mc:Choice>
-      <mc:Fallback>
+      <mc:Fallback xmlns="">
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
             <xdr:cNvPr id="2" name="CuadroTexto 6">
@@ -3176,8 +3176,8 @@
       <xdr:row>36</xdr:row>
       <xdr:rowOff>42093</xdr:rowOff>
     </xdr:to>
-    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-      <mc:Choice xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" Requires="a14">
+    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+      <mc:Choice Requires="a14">
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
             <xdr:cNvPr id="3" name="CuadroTexto 6">
@@ -3354,7 +3354,7 @@
           </xdr:txBody>
         </xdr:sp>
       </mc:Choice>
-      <mc:Fallback>
+      <mc:Fallback xmlns="">
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
             <xdr:cNvPr id="3" name="CuadroTexto 6">
@@ -3491,982 +3491,6 @@
                 <a:t>𝜇+𝑧𝜎</a:t>
               </a:r>
               <a:endParaRPr lang="es-CO" sz="1600"/>
-            </a:p>
-          </xdr:txBody>
-        </xdr:sp>
-      </mc:Fallback>
-    </mc:AlternateContent>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor>
-    <xdr:from>
-      <xdr:col>4</xdr:col>
-      <xdr:colOff>255986</xdr:colOff>
-      <xdr:row>54</xdr:row>
-      <xdr:rowOff>11907</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>8</xdr:col>
-      <xdr:colOff>130970</xdr:colOff>
-      <xdr:row>55</xdr:row>
-      <xdr:rowOff>169367</xdr:rowOff>
-    </xdr:to>
-    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-      <mc:Choice xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" Requires="a14">
-        <xdr:sp macro="" textlink="">
-          <xdr:nvSpPr>
-            <xdr:cNvPr id="4" name="CuadroTexto 12">
-              <a:extLst>
-                <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{B90DAD71-7070-4A89-AA2E-6D2AF79E17E0}"/>
-                </a:ext>
-              </a:extLst>
-            </xdr:cNvPr>
-            <xdr:cNvSpPr txBox="1"/>
-          </xdr:nvSpPr>
-          <xdr:spPr>
-            <a:xfrm>
-              <a:off x="5286377" y="9727407"/>
-              <a:ext cx="2922984" cy="336054"/>
-            </a:xfrm>
-            <a:prstGeom prst="rect">
-              <a:avLst/>
-            </a:prstGeom>
-          </xdr:spPr>
-          <xdr:txBody>
-            <a:bodyPr vert="horz" wrap="square" lIns="91440" tIns="45720" rIns="91440" bIns="45720" rtlCol="0">
-              <a:spAutoFit/>
-            </a:bodyPr>
-            <a:lstStyle>
-              <a:defPPr>
-                <a:defRPr lang="es-CO"/>
-              </a:defPPr>
-              <a:lvl1pPr marL="0" algn="l" defTabSz="914400" rtl="0" eaLnBrk="1" latinLnBrk="0" hangingPunct="1">
-                <a:defRPr sz="1800" kern="1200">
-                  <a:solidFill>
-                    <a:schemeClr val="tx1"/>
-                  </a:solidFill>
-                  <a:latin typeface="+mn-lt"/>
-                  <a:ea typeface="+mn-ea"/>
-                  <a:cs typeface="+mn-cs"/>
-                </a:defRPr>
-              </a:lvl1pPr>
-              <a:lvl2pPr marL="457200" algn="l" defTabSz="914400" rtl="0" eaLnBrk="1" latinLnBrk="0" hangingPunct="1">
-                <a:defRPr sz="1800" kern="1200">
-                  <a:solidFill>
-                    <a:schemeClr val="tx1"/>
-                  </a:solidFill>
-                  <a:latin typeface="+mn-lt"/>
-                  <a:ea typeface="+mn-ea"/>
-                  <a:cs typeface="+mn-cs"/>
-                </a:defRPr>
-              </a:lvl2pPr>
-              <a:lvl3pPr marL="914400" algn="l" defTabSz="914400" rtl="0" eaLnBrk="1" latinLnBrk="0" hangingPunct="1">
-                <a:defRPr sz="1800" kern="1200">
-                  <a:solidFill>
-                    <a:schemeClr val="tx1"/>
-                  </a:solidFill>
-                  <a:latin typeface="+mn-lt"/>
-                  <a:ea typeface="+mn-ea"/>
-                  <a:cs typeface="+mn-cs"/>
-                </a:defRPr>
-              </a:lvl3pPr>
-              <a:lvl4pPr marL="1371600" algn="l" defTabSz="914400" rtl="0" eaLnBrk="1" latinLnBrk="0" hangingPunct="1">
-                <a:defRPr sz="1800" kern="1200">
-                  <a:solidFill>
-                    <a:schemeClr val="tx1"/>
-                  </a:solidFill>
-                  <a:latin typeface="+mn-lt"/>
-                  <a:ea typeface="+mn-ea"/>
-                  <a:cs typeface="+mn-cs"/>
-                </a:defRPr>
-              </a:lvl4pPr>
-              <a:lvl5pPr marL="1828800" algn="l" defTabSz="914400" rtl="0" eaLnBrk="1" latinLnBrk="0" hangingPunct="1">
-                <a:defRPr sz="1800" kern="1200">
-                  <a:solidFill>
-                    <a:schemeClr val="tx1"/>
-                  </a:solidFill>
-                  <a:latin typeface="+mn-lt"/>
-                  <a:ea typeface="+mn-ea"/>
-                  <a:cs typeface="+mn-cs"/>
-                </a:defRPr>
-              </a:lvl5pPr>
-              <a:lvl6pPr marL="2286000" algn="l" defTabSz="914400" rtl="0" eaLnBrk="1" latinLnBrk="0" hangingPunct="1">
-                <a:defRPr sz="1800" kern="1200">
-                  <a:solidFill>
-                    <a:schemeClr val="tx1"/>
-                  </a:solidFill>
-                  <a:latin typeface="+mn-lt"/>
-                  <a:ea typeface="+mn-ea"/>
-                  <a:cs typeface="+mn-cs"/>
-                </a:defRPr>
-              </a:lvl6pPr>
-              <a:lvl7pPr marL="2743200" algn="l" defTabSz="914400" rtl="0" eaLnBrk="1" latinLnBrk="0" hangingPunct="1">
-                <a:defRPr sz="1800" kern="1200">
-                  <a:solidFill>
-                    <a:schemeClr val="tx1"/>
-                  </a:solidFill>
-                  <a:latin typeface="+mn-lt"/>
-                  <a:ea typeface="+mn-ea"/>
-                  <a:cs typeface="+mn-cs"/>
-                </a:defRPr>
-              </a:lvl7pPr>
-              <a:lvl8pPr marL="3200400" algn="l" defTabSz="914400" rtl="0" eaLnBrk="1" latinLnBrk="0" hangingPunct="1">
-                <a:defRPr sz="1800" kern="1200">
-                  <a:solidFill>
-                    <a:schemeClr val="tx1"/>
-                  </a:solidFill>
-                  <a:latin typeface="+mn-lt"/>
-                  <a:ea typeface="+mn-ea"/>
-                  <a:cs typeface="+mn-cs"/>
-                </a:defRPr>
-              </a:lvl8pPr>
-              <a:lvl9pPr marL="3657600" algn="l" defTabSz="914400" rtl="0" eaLnBrk="1" latinLnBrk="0" hangingPunct="1">
-                <a:defRPr sz="1800" kern="1200">
-                  <a:solidFill>
-                    <a:schemeClr val="tx1"/>
-                  </a:solidFill>
-                  <a:latin typeface="+mn-lt"/>
-                  <a:ea typeface="+mn-ea"/>
-                  <a:cs typeface="+mn-cs"/>
-                </a:defRPr>
-              </a:lvl9pPr>
-            </a:lstStyle>
-            <a:p>
-              <a:r>
-                <a:rPr lang="es-MX" sz="1050"/>
-                <a:t>x = a + </a:t>
-              </a:r>
-              <a14:m>
-                <m:oMath xmlns:m="http://schemas.openxmlformats.org/officeDocument/2006/math">
-                  <m:rad>
-                    <m:radPr>
-                      <m:degHide m:val="on"/>
-                      <m:ctrlPr>
-                        <a:rPr lang="es-MX" sz="1050" i="1">
-                          <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
-                        </a:rPr>
-                      </m:ctrlPr>
-                    </m:radPr>
-                    <m:deg/>
-                    <m:e>
-                      <m:r>
-                        <a:rPr lang="es-MX" sz="1050" b="0" i="1">
-                          <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
-                        </a:rPr>
-                        <m:t>𝑃</m:t>
-                      </m:r>
-                      <m:d>
-                        <m:dPr>
-                          <m:ctrlPr>
-                            <a:rPr lang="es-MX" sz="1050" b="0" i="1">
-                              <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
-                            </a:rPr>
-                          </m:ctrlPr>
-                        </m:dPr>
-                        <m:e>
-                          <m:r>
-                            <a:rPr lang="es-MX" sz="1050" b="0" i="1">
-                              <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
-                            </a:rPr>
-                            <m:t>&lt;</m:t>
-                          </m:r>
-                          <m:r>
-                            <a:rPr lang="es-MX" sz="1050" b="0" i="1">
-                              <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
-                            </a:rPr>
-                            <m:t>𝑥</m:t>
-                          </m:r>
-                        </m:e>
-                      </m:d>
-                      <m:r>
-                        <a:rPr lang="es-MX" sz="1050" b="0" i="1">
-                          <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
-                        </a:rPr>
-                        <m:t>𝑏</m:t>
-                      </m:r>
-                      <m:r>
-                        <a:rPr lang="es-MX" sz="1050" b="0" i="1">
-                          <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
-                        </a:rPr>
-                        <m:t>(</m:t>
-                      </m:r>
-                      <m:r>
-                        <a:rPr lang="es-MX" sz="1050" b="0" i="1">
-                          <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
-                        </a:rPr>
-                        <m:t>𝑐</m:t>
-                      </m:r>
-                      <m:r>
-                        <a:rPr lang="es-MX" sz="1050" b="0" i="1">
-                          <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
-                        </a:rPr>
-                        <m:t>−</m:t>
-                      </m:r>
-                      <m:r>
-                        <a:rPr lang="es-MX" sz="1050" b="0" i="1">
-                          <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
-                        </a:rPr>
-                        <m:t>𝑎</m:t>
-                      </m:r>
-                      <m:r>
-                        <a:rPr lang="es-MX" sz="1050" b="0" i="1">
-                          <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
-                        </a:rPr>
-                        <m:t>)</m:t>
-                      </m:r>
-                    </m:e>
-                  </m:rad>
-                </m:oMath>
-              </a14:m>
-              <a:r>
-                <a:rPr lang="es-CO" sz="1050"/>
-                <a:t>, si </a:t>
-              </a:r>
-              <a14:m>
-                <m:oMath xmlns:m="http://schemas.openxmlformats.org/officeDocument/2006/math">
-                  <m:r>
-                    <a:rPr lang="es-MX" sz="1050" b="0" i="1">
-                      <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
-                    </a:rPr>
-                    <m:t>𝑃</m:t>
-                  </m:r>
-                  <m:r>
-                    <a:rPr lang="es-MX" sz="1050" b="0" i="1">
-                      <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
-                    </a:rPr>
-                    <m:t>(&lt;</m:t>
-                  </m:r>
-                  <m:r>
-                    <a:rPr lang="es-MX" sz="1050" b="0" i="1">
-                      <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
-                    </a:rPr>
-                    <m:t>𝑥</m:t>
-                  </m:r>
-                  <m:r>
-                    <a:rPr lang="es-MX" sz="1050" b="0" i="1">
-                      <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
-                    </a:rPr>
-                    <m:t>)≤</m:t>
-                  </m:r>
-                  <m:f>
-                    <m:fPr>
-                      <m:ctrlPr>
-                        <a:rPr lang="es-MX" sz="1050" b="0" i="1">
-                          <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
-                          <a:ea typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
-                        </a:rPr>
-                      </m:ctrlPr>
-                    </m:fPr>
-                    <m:num>
-                      <m:r>
-                        <a:rPr lang="es-MX" sz="1050" b="0" i="1">
-                          <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
-                          <a:ea typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
-                        </a:rPr>
-                        <m:t>𝑏</m:t>
-                      </m:r>
-                      <m:r>
-                        <a:rPr lang="es-MX" sz="1050" b="0" i="1">
-                          <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
-                          <a:ea typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
-                        </a:rPr>
-                        <m:t>−</m:t>
-                      </m:r>
-                      <m:r>
-                        <a:rPr lang="es-MX" sz="1050" b="0" i="1">
-                          <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
-                          <a:ea typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
-                        </a:rPr>
-                        <m:t>𝑎</m:t>
-                      </m:r>
-                    </m:num>
-                    <m:den>
-                      <m:r>
-                        <a:rPr lang="es-MX" sz="1050" b="0" i="1">
-                          <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
-                          <a:ea typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
-                        </a:rPr>
-                        <m:t>𝑐</m:t>
-                      </m:r>
-                      <m:r>
-                        <a:rPr lang="es-MX" sz="1050" b="0" i="1">
-                          <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
-                          <a:ea typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
-                        </a:rPr>
-                        <m:t>−</m:t>
-                      </m:r>
-                      <m:r>
-                        <a:rPr lang="es-MX" sz="1050" b="0" i="1">
-                          <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
-                          <a:ea typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
-                        </a:rPr>
-                        <m:t>𝑎</m:t>
-                      </m:r>
-                    </m:den>
-                  </m:f>
-                </m:oMath>
-              </a14:m>
-              <a:endParaRPr lang="es-CO" sz="1050"/>
-            </a:p>
-          </xdr:txBody>
-        </xdr:sp>
-      </mc:Choice>
-      <mc:Fallback>
-        <xdr:sp macro="" textlink="">
-          <xdr:nvSpPr>
-            <xdr:cNvPr id="4" name="CuadroTexto 12">
-              <a:extLst>
-                <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{B90DAD71-7070-4A89-AA2E-6D2AF79E17E0}"/>
-                </a:ext>
-              </a:extLst>
-            </xdr:cNvPr>
-            <xdr:cNvSpPr txBox="1"/>
-          </xdr:nvSpPr>
-          <xdr:spPr>
-            <a:xfrm>
-              <a:off x="5286377" y="9727407"/>
-              <a:ext cx="2922984" cy="336054"/>
-            </a:xfrm>
-            <a:prstGeom prst="rect">
-              <a:avLst/>
-            </a:prstGeom>
-          </xdr:spPr>
-          <xdr:txBody>
-            <a:bodyPr vert="horz" wrap="square" lIns="91440" tIns="45720" rIns="91440" bIns="45720" rtlCol="0">
-              <a:spAutoFit/>
-            </a:bodyPr>
-            <a:lstStyle>
-              <a:defPPr>
-                <a:defRPr lang="es-CO"/>
-              </a:defPPr>
-              <a:lvl1pPr marL="0" algn="l" defTabSz="914400" rtl="0" eaLnBrk="1" latinLnBrk="0" hangingPunct="1">
-                <a:defRPr sz="1800" kern="1200">
-                  <a:solidFill>
-                    <a:schemeClr val="tx1"/>
-                  </a:solidFill>
-                  <a:latin typeface="+mn-lt"/>
-                  <a:ea typeface="+mn-ea"/>
-                  <a:cs typeface="+mn-cs"/>
-                </a:defRPr>
-              </a:lvl1pPr>
-              <a:lvl2pPr marL="457200" algn="l" defTabSz="914400" rtl="0" eaLnBrk="1" latinLnBrk="0" hangingPunct="1">
-                <a:defRPr sz="1800" kern="1200">
-                  <a:solidFill>
-                    <a:schemeClr val="tx1"/>
-                  </a:solidFill>
-                  <a:latin typeface="+mn-lt"/>
-                  <a:ea typeface="+mn-ea"/>
-                  <a:cs typeface="+mn-cs"/>
-                </a:defRPr>
-              </a:lvl2pPr>
-              <a:lvl3pPr marL="914400" algn="l" defTabSz="914400" rtl="0" eaLnBrk="1" latinLnBrk="0" hangingPunct="1">
-                <a:defRPr sz="1800" kern="1200">
-                  <a:solidFill>
-                    <a:schemeClr val="tx1"/>
-                  </a:solidFill>
-                  <a:latin typeface="+mn-lt"/>
-                  <a:ea typeface="+mn-ea"/>
-                  <a:cs typeface="+mn-cs"/>
-                </a:defRPr>
-              </a:lvl3pPr>
-              <a:lvl4pPr marL="1371600" algn="l" defTabSz="914400" rtl="0" eaLnBrk="1" latinLnBrk="0" hangingPunct="1">
-                <a:defRPr sz="1800" kern="1200">
-                  <a:solidFill>
-                    <a:schemeClr val="tx1"/>
-                  </a:solidFill>
-                  <a:latin typeface="+mn-lt"/>
-                  <a:ea typeface="+mn-ea"/>
-                  <a:cs typeface="+mn-cs"/>
-                </a:defRPr>
-              </a:lvl4pPr>
-              <a:lvl5pPr marL="1828800" algn="l" defTabSz="914400" rtl="0" eaLnBrk="1" latinLnBrk="0" hangingPunct="1">
-                <a:defRPr sz="1800" kern="1200">
-                  <a:solidFill>
-                    <a:schemeClr val="tx1"/>
-                  </a:solidFill>
-                  <a:latin typeface="+mn-lt"/>
-                  <a:ea typeface="+mn-ea"/>
-                  <a:cs typeface="+mn-cs"/>
-                </a:defRPr>
-              </a:lvl5pPr>
-              <a:lvl6pPr marL="2286000" algn="l" defTabSz="914400" rtl="0" eaLnBrk="1" latinLnBrk="0" hangingPunct="1">
-                <a:defRPr sz="1800" kern="1200">
-                  <a:solidFill>
-                    <a:schemeClr val="tx1"/>
-                  </a:solidFill>
-                  <a:latin typeface="+mn-lt"/>
-                  <a:ea typeface="+mn-ea"/>
-                  <a:cs typeface="+mn-cs"/>
-                </a:defRPr>
-              </a:lvl6pPr>
-              <a:lvl7pPr marL="2743200" algn="l" defTabSz="914400" rtl="0" eaLnBrk="1" latinLnBrk="0" hangingPunct="1">
-                <a:defRPr sz="1800" kern="1200">
-                  <a:solidFill>
-                    <a:schemeClr val="tx1"/>
-                  </a:solidFill>
-                  <a:latin typeface="+mn-lt"/>
-                  <a:ea typeface="+mn-ea"/>
-                  <a:cs typeface="+mn-cs"/>
-                </a:defRPr>
-              </a:lvl7pPr>
-              <a:lvl8pPr marL="3200400" algn="l" defTabSz="914400" rtl="0" eaLnBrk="1" latinLnBrk="0" hangingPunct="1">
-                <a:defRPr sz="1800" kern="1200">
-                  <a:solidFill>
-                    <a:schemeClr val="tx1"/>
-                  </a:solidFill>
-                  <a:latin typeface="+mn-lt"/>
-                  <a:ea typeface="+mn-ea"/>
-                  <a:cs typeface="+mn-cs"/>
-                </a:defRPr>
-              </a:lvl8pPr>
-              <a:lvl9pPr marL="3657600" algn="l" defTabSz="914400" rtl="0" eaLnBrk="1" latinLnBrk="0" hangingPunct="1">
-                <a:defRPr sz="1800" kern="1200">
-                  <a:solidFill>
-                    <a:schemeClr val="tx1"/>
-                  </a:solidFill>
-                  <a:latin typeface="+mn-lt"/>
-                  <a:ea typeface="+mn-ea"/>
-                  <a:cs typeface="+mn-cs"/>
-                </a:defRPr>
-              </a:lvl9pPr>
-            </a:lstStyle>
-            <a:p>
-              <a:r>
-                <a:rPr lang="es-MX" sz="1050"/>
-                <a:t>x = a + </a:t>
-              </a:r>
-              <a:r>
-                <a:rPr lang="es-MX" sz="1050" i="0">
-                  <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
-                </a:rPr>
-                <a:t>√(</a:t>
-              </a:r>
-              <a:r>
-                <a:rPr lang="es-MX" sz="1050" b="0" i="0">
-                  <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
-                </a:rPr>
-                <a:t>𝑃(&lt;𝑥)𝑏(𝑐−𝑎))</a:t>
-              </a:r>
-              <a:r>
-                <a:rPr lang="es-CO" sz="1050"/>
-                <a:t>, si </a:t>
-              </a:r>
-              <a:r>
-                <a:rPr lang="es-MX" sz="1050" b="0" i="0">
-                  <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
-                </a:rPr>
-                <a:t>𝑃(&lt;𝑥)≤</a:t>
-              </a:r>
-              <a:r>
-                <a:rPr lang="es-MX" sz="1050" b="0" i="0">
-                  <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
-                  <a:ea typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
-                </a:rPr>
-                <a:t>(𝑏−𝑎)/(𝑐−𝑎)</a:t>
-              </a:r>
-              <a:endParaRPr lang="es-CO" sz="1050"/>
-            </a:p>
-          </xdr:txBody>
-        </xdr:sp>
-      </mc:Fallback>
-    </mc:AlternateContent>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor>
-    <xdr:from>
-      <xdr:col>4</xdr:col>
-      <xdr:colOff>244078</xdr:colOff>
-      <xdr:row>56</xdr:row>
-      <xdr:rowOff>10681</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>9</xdr:col>
-      <xdr:colOff>636984</xdr:colOff>
-      <xdr:row>57</xdr:row>
-      <xdr:rowOff>168142</xdr:rowOff>
-    </xdr:to>
-    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-      <mc:Choice xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" Requires="a14">
-        <xdr:sp macro="" textlink="">
-          <xdr:nvSpPr>
-            <xdr:cNvPr id="5" name="CuadroTexto 13">
-              <a:extLst>
-                <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{19471BEB-30F5-48EC-9F1E-46BD46122B63}"/>
-                </a:ext>
-              </a:extLst>
-            </xdr:cNvPr>
-            <xdr:cNvSpPr txBox="1"/>
-          </xdr:nvSpPr>
-          <xdr:spPr>
-            <a:xfrm>
-              <a:off x="5274469" y="10083369"/>
-              <a:ext cx="4202906" cy="336054"/>
-            </a:xfrm>
-            <a:prstGeom prst="rect">
-              <a:avLst/>
-            </a:prstGeom>
-          </xdr:spPr>
-          <xdr:txBody>
-            <a:bodyPr vert="horz" wrap="square" lIns="91440" tIns="45720" rIns="91440" bIns="45720" rtlCol="0">
-              <a:spAutoFit/>
-            </a:bodyPr>
-            <a:lstStyle>
-              <a:defPPr>
-                <a:defRPr lang="es-CO"/>
-              </a:defPPr>
-              <a:lvl1pPr marL="0" algn="l" defTabSz="914400" rtl="0" eaLnBrk="1" latinLnBrk="0" hangingPunct="1">
-                <a:defRPr sz="1800" kern="1200">
-                  <a:solidFill>
-                    <a:schemeClr val="tx1"/>
-                  </a:solidFill>
-                  <a:latin typeface="+mn-lt"/>
-                  <a:ea typeface="+mn-ea"/>
-                  <a:cs typeface="+mn-cs"/>
-                </a:defRPr>
-              </a:lvl1pPr>
-              <a:lvl2pPr marL="457200" algn="l" defTabSz="914400" rtl="0" eaLnBrk="1" latinLnBrk="0" hangingPunct="1">
-                <a:defRPr sz="1800" kern="1200">
-                  <a:solidFill>
-                    <a:schemeClr val="tx1"/>
-                  </a:solidFill>
-                  <a:latin typeface="+mn-lt"/>
-                  <a:ea typeface="+mn-ea"/>
-                  <a:cs typeface="+mn-cs"/>
-                </a:defRPr>
-              </a:lvl2pPr>
-              <a:lvl3pPr marL="914400" algn="l" defTabSz="914400" rtl="0" eaLnBrk="1" latinLnBrk="0" hangingPunct="1">
-                <a:defRPr sz="1800" kern="1200">
-                  <a:solidFill>
-                    <a:schemeClr val="tx1"/>
-                  </a:solidFill>
-                  <a:latin typeface="+mn-lt"/>
-                  <a:ea typeface="+mn-ea"/>
-                  <a:cs typeface="+mn-cs"/>
-                </a:defRPr>
-              </a:lvl3pPr>
-              <a:lvl4pPr marL="1371600" algn="l" defTabSz="914400" rtl="0" eaLnBrk="1" latinLnBrk="0" hangingPunct="1">
-                <a:defRPr sz="1800" kern="1200">
-                  <a:solidFill>
-                    <a:schemeClr val="tx1"/>
-                  </a:solidFill>
-                  <a:latin typeface="+mn-lt"/>
-                  <a:ea typeface="+mn-ea"/>
-                  <a:cs typeface="+mn-cs"/>
-                </a:defRPr>
-              </a:lvl4pPr>
-              <a:lvl5pPr marL="1828800" algn="l" defTabSz="914400" rtl="0" eaLnBrk="1" latinLnBrk="0" hangingPunct="1">
-                <a:defRPr sz="1800" kern="1200">
-                  <a:solidFill>
-                    <a:schemeClr val="tx1"/>
-                  </a:solidFill>
-                  <a:latin typeface="+mn-lt"/>
-                  <a:ea typeface="+mn-ea"/>
-                  <a:cs typeface="+mn-cs"/>
-                </a:defRPr>
-              </a:lvl5pPr>
-              <a:lvl6pPr marL="2286000" algn="l" defTabSz="914400" rtl="0" eaLnBrk="1" latinLnBrk="0" hangingPunct="1">
-                <a:defRPr sz="1800" kern="1200">
-                  <a:solidFill>
-                    <a:schemeClr val="tx1"/>
-                  </a:solidFill>
-                  <a:latin typeface="+mn-lt"/>
-                  <a:ea typeface="+mn-ea"/>
-                  <a:cs typeface="+mn-cs"/>
-                </a:defRPr>
-              </a:lvl6pPr>
-              <a:lvl7pPr marL="2743200" algn="l" defTabSz="914400" rtl="0" eaLnBrk="1" latinLnBrk="0" hangingPunct="1">
-                <a:defRPr sz="1800" kern="1200">
-                  <a:solidFill>
-                    <a:schemeClr val="tx1"/>
-                  </a:solidFill>
-                  <a:latin typeface="+mn-lt"/>
-                  <a:ea typeface="+mn-ea"/>
-                  <a:cs typeface="+mn-cs"/>
-                </a:defRPr>
-              </a:lvl7pPr>
-              <a:lvl8pPr marL="3200400" algn="l" defTabSz="914400" rtl="0" eaLnBrk="1" latinLnBrk="0" hangingPunct="1">
-                <a:defRPr sz="1800" kern="1200">
-                  <a:solidFill>
-                    <a:schemeClr val="tx1"/>
-                  </a:solidFill>
-                  <a:latin typeface="+mn-lt"/>
-                  <a:ea typeface="+mn-ea"/>
-                  <a:cs typeface="+mn-cs"/>
-                </a:defRPr>
-              </a:lvl8pPr>
-              <a:lvl9pPr marL="3657600" algn="l" defTabSz="914400" rtl="0" eaLnBrk="1" latinLnBrk="0" hangingPunct="1">
-                <a:defRPr sz="1800" kern="1200">
-                  <a:solidFill>
-                    <a:schemeClr val="tx1"/>
-                  </a:solidFill>
-                  <a:latin typeface="+mn-lt"/>
-                  <a:ea typeface="+mn-ea"/>
-                  <a:cs typeface="+mn-cs"/>
-                </a:defRPr>
-              </a:lvl9pPr>
-            </a:lstStyle>
-            <a:p>
-              <a:r>
-                <a:rPr lang="es-MX" sz="1050"/>
-                <a:t>x = c + </a:t>
-              </a:r>
-              <a14:m>
-                <m:oMath xmlns:m="http://schemas.openxmlformats.org/officeDocument/2006/math">
-                  <m:rad>
-                    <m:radPr>
-                      <m:degHide m:val="on"/>
-                      <m:ctrlPr>
-                        <a:rPr lang="es-MX" sz="1050" i="1">
-                          <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
-                        </a:rPr>
-                      </m:ctrlPr>
-                    </m:radPr>
-                    <m:deg/>
-                    <m:e>
-                      <m:r>
-                        <a:rPr lang="es-MX" sz="1050" b="0" i="1">
-                          <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
-                        </a:rPr>
-                        <m:t>[1−</m:t>
-                      </m:r>
-                      <m:r>
-                        <a:rPr lang="es-MX" sz="1050" b="0" i="1">
-                          <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
-                        </a:rPr>
-                        <m:t>𝑃</m:t>
-                      </m:r>
-                      <m:d>
-                        <m:dPr>
-                          <m:ctrlPr>
-                            <a:rPr lang="es-MX" sz="1050" b="0" i="1">
-                              <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
-                            </a:rPr>
-                          </m:ctrlPr>
-                        </m:dPr>
-                        <m:e>
-                          <m:r>
-                            <a:rPr lang="es-MX" sz="1050" b="0" i="1">
-                              <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
-                            </a:rPr>
-                            <m:t>&lt;</m:t>
-                          </m:r>
-                          <m:r>
-                            <a:rPr lang="es-MX" sz="1050" b="0" i="1">
-                              <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
-                            </a:rPr>
-                            <m:t>𝑥</m:t>
-                          </m:r>
-                        </m:e>
-                      </m:d>
-                      <m:r>
-                        <a:rPr lang="es-MX" sz="1050" b="0" i="1">
-                          <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
-                        </a:rPr>
-                        <m:t>](</m:t>
-                      </m:r>
-                      <m:r>
-                        <a:rPr lang="es-MX" sz="1050" b="0" i="1">
-                          <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
-                        </a:rPr>
-                        <m:t>𝑏</m:t>
-                      </m:r>
-                      <m:r>
-                        <a:rPr lang="es-MX" sz="1050" b="0" i="1">
-                          <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
-                        </a:rPr>
-                        <m:t>−</m:t>
-                      </m:r>
-                      <m:r>
-                        <a:rPr lang="es-MX" sz="1050" b="0" i="1">
-                          <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
-                        </a:rPr>
-                        <m:t>𝑎</m:t>
-                      </m:r>
-                      <m:r>
-                        <a:rPr lang="es-MX" sz="1050" b="0" i="1">
-                          <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
-                        </a:rPr>
-                        <m:t>)(</m:t>
-                      </m:r>
-                      <m:r>
-                        <a:rPr lang="es-MX" sz="1050" b="0" i="1">
-                          <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
-                        </a:rPr>
-                        <m:t>𝑐</m:t>
-                      </m:r>
-                      <m:r>
-                        <a:rPr lang="es-MX" sz="1050" b="0" i="1">
-                          <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
-                        </a:rPr>
-                        <m:t>−</m:t>
-                      </m:r>
-                      <m:r>
-                        <a:rPr lang="es-MX" sz="1050" b="0" i="1">
-                          <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
-                        </a:rPr>
-                        <m:t>𝑎</m:t>
-                      </m:r>
-                      <m:r>
-                        <a:rPr lang="es-MX" sz="1050" b="0" i="1">
-                          <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
-                        </a:rPr>
-                        <m:t>)</m:t>
-                      </m:r>
-                    </m:e>
-                  </m:rad>
-                </m:oMath>
-              </a14:m>
-              <a:r>
-                <a:rPr lang="es-CO" sz="1050"/>
-                <a:t>, si </a:t>
-              </a:r>
-              <a14:m>
-                <m:oMath xmlns:m="http://schemas.openxmlformats.org/officeDocument/2006/math">
-                  <m:r>
-                    <a:rPr lang="es-MX" sz="1050" b="0" i="1">
-                      <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
-                    </a:rPr>
-                    <m:t>𝑃</m:t>
-                  </m:r>
-                  <m:r>
-                    <a:rPr lang="es-MX" sz="1050" b="0" i="1">
-                      <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
-                    </a:rPr>
-                    <m:t>(&lt;</m:t>
-                  </m:r>
-                  <m:r>
-                    <a:rPr lang="es-MX" sz="1050" b="0" i="1">
-                      <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
-                    </a:rPr>
-                    <m:t>𝑥</m:t>
-                  </m:r>
-                  <m:r>
-                    <a:rPr lang="es-MX" sz="1050" b="0" i="1">
-                      <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
-                    </a:rPr>
-                    <m:t>)&gt;</m:t>
-                  </m:r>
-                  <m:f>
-                    <m:fPr>
-                      <m:ctrlPr>
-                        <a:rPr lang="es-MX" sz="1050" b="0" i="1">
-                          <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
-                          <a:ea typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
-                        </a:rPr>
-                      </m:ctrlPr>
-                    </m:fPr>
-                    <m:num>
-                      <m:r>
-                        <a:rPr lang="es-MX" sz="1050" b="0" i="1">
-                          <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
-                          <a:ea typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
-                        </a:rPr>
-                        <m:t>𝑏</m:t>
-                      </m:r>
-                      <m:r>
-                        <a:rPr lang="es-MX" sz="1050" b="0" i="1">
-                          <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
-                          <a:ea typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
-                        </a:rPr>
-                        <m:t>−</m:t>
-                      </m:r>
-                      <m:r>
-                        <a:rPr lang="es-MX" sz="1050" b="0" i="1">
-                          <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
-                          <a:ea typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
-                        </a:rPr>
-                        <m:t>𝑎</m:t>
-                      </m:r>
-                    </m:num>
-                    <m:den>
-                      <m:r>
-                        <a:rPr lang="es-MX" sz="1050" b="0" i="1">
-                          <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
-                          <a:ea typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
-                        </a:rPr>
-                        <m:t>𝑐</m:t>
-                      </m:r>
-                      <m:r>
-                        <a:rPr lang="es-MX" sz="1050" b="0" i="1">
-                          <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
-                          <a:ea typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
-                        </a:rPr>
-                        <m:t>−</m:t>
-                      </m:r>
-                      <m:r>
-                        <a:rPr lang="es-MX" sz="1050" b="0" i="1">
-                          <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
-                          <a:ea typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
-                        </a:rPr>
-                        <m:t>𝑎</m:t>
-                      </m:r>
-                    </m:den>
-                  </m:f>
-                </m:oMath>
-              </a14:m>
-              <a:endParaRPr lang="es-CO" sz="1050"/>
-            </a:p>
-          </xdr:txBody>
-        </xdr:sp>
-      </mc:Choice>
-      <mc:Fallback>
-        <xdr:sp macro="" textlink="">
-          <xdr:nvSpPr>
-            <xdr:cNvPr id="5" name="CuadroTexto 13">
-              <a:extLst>
-                <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{19471BEB-30F5-48EC-9F1E-46BD46122B63}"/>
-                </a:ext>
-              </a:extLst>
-            </xdr:cNvPr>
-            <xdr:cNvSpPr txBox="1"/>
-          </xdr:nvSpPr>
-          <xdr:spPr>
-            <a:xfrm>
-              <a:off x="5274469" y="10083369"/>
-              <a:ext cx="4202906" cy="336054"/>
-            </a:xfrm>
-            <a:prstGeom prst="rect">
-              <a:avLst/>
-            </a:prstGeom>
-          </xdr:spPr>
-          <xdr:txBody>
-            <a:bodyPr vert="horz" wrap="square" lIns="91440" tIns="45720" rIns="91440" bIns="45720" rtlCol="0">
-              <a:spAutoFit/>
-            </a:bodyPr>
-            <a:lstStyle>
-              <a:defPPr>
-                <a:defRPr lang="es-CO"/>
-              </a:defPPr>
-              <a:lvl1pPr marL="0" algn="l" defTabSz="914400" rtl="0" eaLnBrk="1" latinLnBrk="0" hangingPunct="1">
-                <a:defRPr sz="1800" kern="1200">
-                  <a:solidFill>
-                    <a:schemeClr val="tx1"/>
-                  </a:solidFill>
-                  <a:latin typeface="+mn-lt"/>
-                  <a:ea typeface="+mn-ea"/>
-                  <a:cs typeface="+mn-cs"/>
-                </a:defRPr>
-              </a:lvl1pPr>
-              <a:lvl2pPr marL="457200" algn="l" defTabSz="914400" rtl="0" eaLnBrk="1" latinLnBrk="0" hangingPunct="1">
-                <a:defRPr sz="1800" kern="1200">
-                  <a:solidFill>
-                    <a:schemeClr val="tx1"/>
-                  </a:solidFill>
-                  <a:latin typeface="+mn-lt"/>
-                  <a:ea typeface="+mn-ea"/>
-                  <a:cs typeface="+mn-cs"/>
-                </a:defRPr>
-              </a:lvl2pPr>
-              <a:lvl3pPr marL="914400" algn="l" defTabSz="914400" rtl="0" eaLnBrk="1" latinLnBrk="0" hangingPunct="1">
-                <a:defRPr sz="1800" kern="1200">
-                  <a:solidFill>
-                    <a:schemeClr val="tx1"/>
-                  </a:solidFill>
-                  <a:latin typeface="+mn-lt"/>
-                  <a:ea typeface="+mn-ea"/>
-                  <a:cs typeface="+mn-cs"/>
-                </a:defRPr>
-              </a:lvl3pPr>
-              <a:lvl4pPr marL="1371600" algn="l" defTabSz="914400" rtl="0" eaLnBrk="1" latinLnBrk="0" hangingPunct="1">
-                <a:defRPr sz="1800" kern="1200">
-                  <a:solidFill>
-                    <a:schemeClr val="tx1"/>
-                  </a:solidFill>
-                  <a:latin typeface="+mn-lt"/>
-                  <a:ea typeface="+mn-ea"/>
-                  <a:cs typeface="+mn-cs"/>
-                </a:defRPr>
-              </a:lvl4pPr>
-              <a:lvl5pPr marL="1828800" algn="l" defTabSz="914400" rtl="0" eaLnBrk="1" latinLnBrk="0" hangingPunct="1">
-                <a:defRPr sz="1800" kern="1200">
-                  <a:solidFill>
-                    <a:schemeClr val="tx1"/>
-                  </a:solidFill>
-                  <a:latin typeface="+mn-lt"/>
-                  <a:ea typeface="+mn-ea"/>
-                  <a:cs typeface="+mn-cs"/>
-                </a:defRPr>
-              </a:lvl5pPr>
-              <a:lvl6pPr marL="2286000" algn="l" defTabSz="914400" rtl="0" eaLnBrk="1" latinLnBrk="0" hangingPunct="1">
-                <a:defRPr sz="1800" kern="1200">
-                  <a:solidFill>
-                    <a:schemeClr val="tx1"/>
-                  </a:solidFill>
-                  <a:latin typeface="+mn-lt"/>
-                  <a:ea typeface="+mn-ea"/>
-                  <a:cs typeface="+mn-cs"/>
-                </a:defRPr>
-              </a:lvl6pPr>
-              <a:lvl7pPr marL="2743200" algn="l" defTabSz="914400" rtl="0" eaLnBrk="1" latinLnBrk="0" hangingPunct="1">
-                <a:defRPr sz="1800" kern="1200">
-                  <a:solidFill>
-                    <a:schemeClr val="tx1"/>
-                  </a:solidFill>
-                  <a:latin typeface="+mn-lt"/>
-                  <a:ea typeface="+mn-ea"/>
-                  <a:cs typeface="+mn-cs"/>
-                </a:defRPr>
-              </a:lvl7pPr>
-              <a:lvl8pPr marL="3200400" algn="l" defTabSz="914400" rtl="0" eaLnBrk="1" latinLnBrk="0" hangingPunct="1">
-                <a:defRPr sz="1800" kern="1200">
-                  <a:solidFill>
-                    <a:schemeClr val="tx1"/>
-                  </a:solidFill>
-                  <a:latin typeface="+mn-lt"/>
-                  <a:ea typeface="+mn-ea"/>
-                  <a:cs typeface="+mn-cs"/>
-                </a:defRPr>
-              </a:lvl8pPr>
-              <a:lvl9pPr marL="3657600" algn="l" defTabSz="914400" rtl="0" eaLnBrk="1" latinLnBrk="0" hangingPunct="1">
-                <a:defRPr sz="1800" kern="1200">
-                  <a:solidFill>
-                    <a:schemeClr val="tx1"/>
-                  </a:solidFill>
-                  <a:latin typeface="+mn-lt"/>
-                  <a:ea typeface="+mn-ea"/>
-                  <a:cs typeface="+mn-cs"/>
-                </a:defRPr>
-              </a:lvl9pPr>
-            </a:lstStyle>
-            <a:p>
-              <a:r>
-                <a:rPr lang="es-MX" sz="1050"/>
-                <a:t>x = c + </a:t>
-              </a:r>
-              <a:r>
-                <a:rPr lang="es-MX" sz="1050" i="0">
-                  <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
-                </a:rPr>
-                <a:t>√(</a:t>
-              </a:r>
-              <a:r>
-                <a:rPr lang="es-MX" sz="1050" b="0" i="0">
-                  <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
-                </a:rPr>
-                <a:t>[1−𝑃(&lt;𝑥)](𝑏−𝑎)(𝑐−𝑎))</a:t>
-              </a:r>
-              <a:r>
-                <a:rPr lang="es-CO" sz="1050"/>
-                <a:t>, si </a:t>
-              </a:r>
-              <a:r>
-                <a:rPr lang="es-MX" sz="1050" b="0" i="0">
-                  <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
-                </a:rPr>
-                <a:t>𝑃(&lt;𝑥)&gt;</a:t>
-              </a:r>
-              <a:r>
-                <a:rPr lang="es-MX" sz="1050" b="0" i="0">
-                  <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
-                  <a:ea typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
-                </a:rPr>
-                <a:t>(𝑏−𝑎)/(𝑐−𝑎)</a:t>
-              </a:r>
-              <a:endParaRPr lang="es-CO" sz="1050"/>
             </a:p>
           </xdr:txBody>
         </xdr:sp>
@@ -4695,6 +3719,1037 @@
         </a:p>
       </xdr:txBody>
     </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>3</xdr:col>
+      <xdr:colOff>270056</xdr:colOff>
+      <xdr:row>54</xdr:row>
+      <xdr:rowOff>83343</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>6</xdr:col>
+      <xdr:colOff>581458</xdr:colOff>
+      <xdr:row>56</xdr:row>
+      <xdr:rowOff>18030</xdr:rowOff>
+    </xdr:to>
+    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+      <mc:Choice xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" Requires="a14">
+        <xdr:sp macro="" textlink="">
+          <xdr:nvSpPr>
+            <xdr:cNvPr id="8" name="CuadroTexto 12">
+              <a:extLst>
+                <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{4E34FD70-1C53-4FDC-8875-98645C53E3B7}"/>
+                </a:ext>
+              </a:extLst>
+            </xdr:cNvPr>
+            <xdr:cNvSpPr txBox="1"/>
+          </xdr:nvSpPr>
+          <xdr:spPr>
+            <a:xfrm>
+              <a:off x="4080056" y="9798843"/>
+              <a:ext cx="3055793" cy="291875"/>
+            </a:xfrm>
+            <a:prstGeom prst="rect">
+              <a:avLst/>
+            </a:prstGeom>
+          </xdr:spPr>
+          <xdr:txBody>
+            <a:bodyPr vert="horz" wrap="square" lIns="91440" tIns="45720" rIns="91440" bIns="45720" rtlCol="0">
+              <a:spAutoFit/>
+            </a:bodyPr>
+            <a:lstStyle>
+              <a:defPPr>
+                <a:defRPr lang="es-CO"/>
+              </a:defPPr>
+              <a:lvl1pPr marL="0" algn="l" defTabSz="914400" rtl="0" eaLnBrk="1" latinLnBrk="0" hangingPunct="1">
+                <a:defRPr sz="1800" kern="1200">
+                  <a:solidFill>
+                    <a:schemeClr val="tx1"/>
+                  </a:solidFill>
+                  <a:latin typeface="+mn-lt"/>
+                  <a:ea typeface="+mn-ea"/>
+                  <a:cs typeface="+mn-cs"/>
+                </a:defRPr>
+              </a:lvl1pPr>
+              <a:lvl2pPr marL="457200" algn="l" defTabSz="914400" rtl="0" eaLnBrk="1" latinLnBrk="0" hangingPunct="1">
+                <a:defRPr sz="1800" kern="1200">
+                  <a:solidFill>
+                    <a:schemeClr val="tx1"/>
+                  </a:solidFill>
+                  <a:latin typeface="+mn-lt"/>
+                  <a:ea typeface="+mn-ea"/>
+                  <a:cs typeface="+mn-cs"/>
+                </a:defRPr>
+              </a:lvl2pPr>
+              <a:lvl3pPr marL="914400" algn="l" defTabSz="914400" rtl="0" eaLnBrk="1" latinLnBrk="0" hangingPunct="1">
+                <a:defRPr sz="1800" kern="1200">
+                  <a:solidFill>
+                    <a:schemeClr val="tx1"/>
+                  </a:solidFill>
+                  <a:latin typeface="+mn-lt"/>
+                  <a:ea typeface="+mn-ea"/>
+                  <a:cs typeface="+mn-cs"/>
+                </a:defRPr>
+              </a:lvl3pPr>
+              <a:lvl4pPr marL="1371600" algn="l" defTabSz="914400" rtl="0" eaLnBrk="1" latinLnBrk="0" hangingPunct="1">
+                <a:defRPr sz="1800" kern="1200">
+                  <a:solidFill>
+                    <a:schemeClr val="tx1"/>
+                  </a:solidFill>
+                  <a:latin typeface="+mn-lt"/>
+                  <a:ea typeface="+mn-ea"/>
+                  <a:cs typeface="+mn-cs"/>
+                </a:defRPr>
+              </a:lvl4pPr>
+              <a:lvl5pPr marL="1828800" algn="l" defTabSz="914400" rtl="0" eaLnBrk="1" latinLnBrk="0" hangingPunct="1">
+                <a:defRPr sz="1800" kern="1200">
+                  <a:solidFill>
+                    <a:schemeClr val="tx1"/>
+                  </a:solidFill>
+                  <a:latin typeface="+mn-lt"/>
+                  <a:ea typeface="+mn-ea"/>
+                  <a:cs typeface="+mn-cs"/>
+                </a:defRPr>
+              </a:lvl5pPr>
+              <a:lvl6pPr marL="2286000" algn="l" defTabSz="914400" rtl="0" eaLnBrk="1" latinLnBrk="0" hangingPunct="1">
+                <a:defRPr sz="1800" kern="1200">
+                  <a:solidFill>
+                    <a:schemeClr val="tx1"/>
+                  </a:solidFill>
+                  <a:latin typeface="+mn-lt"/>
+                  <a:ea typeface="+mn-ea"/>
+                  <a:cs typeface="+mn-cs"/>
+                </a:defRPr>
+              </a:lvl6pPr>
+              <a:lvl7pPr marL="2743200" algn="l" defTabSz="914400" rtl="0" eaLnBrk="1" latinLnBrk="0" hangingPunct="1">
+                <a:defRPr sz="1800" kern="1200">
+                  <a:solidFill>
+                    <a:schemeClr val="tx1"/>
+                  </a:solidFill>
+                  <a:latin typeface="+mn-lt"/>
+                  <a:ea typeface="+mn-ea"/>
+                  <a:cs typeface="+mn-cs"/>
+                </a:defRPr>
+              </a:lvl7pPr>
+              <a:lvl8pPr marL="3200400" algn="l" defTabSz="914400" rtl="0" eaLnBrk="1" latinLnBrk="0" hangingPunct="1">
+                <a:defRPr sz="1800" kern="1200">
+                  <a:solidFill>
+                    <a:schemeClr val="tx1"/>
+                  </a:solidFill>
+                  <a:latin typeface="+mn-lt"/>
+                  <a:ea typeface="+mn-ea"/>
+                  <a:cs typeface="+mn-cs"/>
+                </a:defRPr>
+              </a:lvl8pPr>
+              <a:lvl9pPr marL="3657600" algn="l" defTabSz="914400" rtl="0" eaLnBrk="1" latinLnBrk="0" hangingPunct="1">
+                <a:defRPr sz="1800" kern="1200">
+                  <a:solidFill>
+                    <a:schemeClr val="tx1"/>
+                  </a:solidFill>
+                  <a:latin typeface="+mn-lt"/>
+                  <a:ea typeface="+mn-ea"/>
+                  <a:cs typeface="+mn-cs"/>
+                </a:defRPr>
+              </a:lvl9pPr>
+            </a:lstStyle>
+            <a:p>
+              <a:r>
+                <a:rPr lang="es-MX" sz="900"/>
+                <a:t>x = a + </a:t>
+              </a:r>
+              <a14:m>
+                <m:oMath xmlns:m="http://schemas.openxmlformats.org/officeDocument/2006/math">
+                  <m:rad>
+                    <m:radPr>
+                      <m:degHide m:val="on"/>
+                      <m:ctrlPr>
+                        <a:rPr lang="es-MX" sz="900" i="1">
+                          <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
+                        </a:rPr>
+                      </m:ctrlPr>
+                    </m:radPr>
+                    <m:deg/>
+                    <m:e>
+                      <m:r>
+                        <a:rPr lang="es-MX" sz="900" b="0" i="1">
+                          <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
+                        </a:rPr>
+                        <m:t>𝑃</m:t>
+                      </m:r>
+                      <m:d>
+                        <m:dPr>
+                          <m:ctrlPr>
+                            <a:rPr lang="es-MX" sz="900" b="0" i="1">
+                              <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
+                            </a:rPr>
+                          </m:ctrlPr>
+                        </m:dPr>
+                        <m:e>
+                          <m:r>
+                            <a:rPr lang="es-MX" sz="900" b="0" i="1">
+                              <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
+                            </a:rPr>
+                            <m:t>&lt;</m:t>
+                          </m:r>
+                          <m:r>
+                            <a:rPr lang="es-MX" sz="900" b="0" i="1">
+                              <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
+                            </a:rPr>
+                            <m:t>𝑥</m:t>
+                          </m:r>
+                        </m:e>
+                      </m:d>
+                      <m:r>
+                        <a:rPr lang="es-MX" sz="900" b="0" i="1">
+                          <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
+                        </a:rPr>
+                        <m:t>(</m:t>
+                      </m:r>
+                      <m:r>
+                        <a:rPr lang="es-MX" sz="900" b="0" i="1">
+                          <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
+                        </a:rPr>
+                        <m:t>𝑏</m:t>
+                      </m:r>
+                      <m:r>
+                        <a:rPr lang="es-MX" sz="900" b="0" i="1">
+                          <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
+                        </a:rPr>
+                        <m:t>−</m:t>
+                      </m:r>
+                      <m:r>
+                        <a:rPr lang="es-MX" sz="900" b="0" i="1">
+                          <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
+                        </a:rPr>
+                        <m:t>𝑎</m:t>
+                      </m:r>
+                      <m:r>
+                        <a:rPr lang="es-MX" sz="900" b="0" i="1">
+                          <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
+                        </a:rPr>
+                        <m:t>)(</m:t>
+                      </m:r>
+                      <m:r>
+                        <a:rPr lang="es-MX" sz="900" b="0" i="1">
+                          <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
+                        </a:rPr>
+                        <m:t>𝑐</m:t>
+                      </m:r>
+                      <m:r>
+                        <a:rPr lang="es-MX" sz="900" b="0" i="1">
+                          <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
+                        </a:rPr>
+                        <m:t>−</m:t>
+                      </m:r>
+                      <m:r>
+                        <a:rPr lang="es-MX" sz="900" b="0" i="1">
+                          <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
+                        </a:rPr>
+                        <m:t>𝑎</m:t>
+                      </m:r>
+                      <m:r>
+                        <a:rPr lang="es-MX" sz="900" b="0" i="1">
+                          <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
+                        </a:rPr>
+                        <m:t>)</m:t>
+                      </m:r>
+                    </m:e>
+                  </m:rad>
+                </m:oMath>
+              </a14:m>
+              <a:r>
+                <a:rPr lang="es-CO" sz="900"/>
+                <a:t>, 	si </a:t>
+              </a:r>
+              <a14:m>
+                <m:oMath xmlns:m="http://schemas.openxmlformats.org/officeDocument/2006/math">
+                  <m:r>
+                    <a:rPr lang="es-MX" sz="900" b="0" i="1">
+                      <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
+                    </a:rPr>
+                    <m:t>𝑃</m:t>
+                  </m:r>
+                  <m:r>
+                    <a:rPr lang="es-MX" sz="900" b="0" i="1">
+                      <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
+                    </a:rPr>
+                    <m:t>(&lt;</m:t>
+                  </m:r>
+                  <m:r>
+                    <a:rPr lang="es-MX" sz="900" b="0" i="1">
+                      <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
+                    </a:rPr>
+                    <m:t>𝑥</m:t>
+                  </m:r>
+                  <m:r>
+                    <a:rPr lang="es-MX" sz="900" b="0" i="1">
+                      <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
+                    </a:rPr>
+                    <m:t>)≤</m:t>
+                  </m:r>
+                  <m:f>
+                    <m:fPr>
+                      <m:ctrlPr>
+                        <a:rPr lang="es-MX" sz="900" b="0" i="1">
+                          <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
+                          <a:ea typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
+                        </a:rPr>
+                      </m:ctrlPr>
+                    </m:fPr>
+                    <m:num>
+                      <m:r>
+                        <a:rPr lang="es-MX" sz="900" b="0" i="1">
+                          <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
+                          <a:ea typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
+                        </a:rPr>
+                        <m:t>𝑏</m:t>
+                      </m:r>
+                      <m:r>
+                        <a:rPr lang="es-MX" sz="900" b="0" i="1">
+                          <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
+                          <a:ea typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
+                        </a:rPr>
+                        <m:t>−</m:t>
+                      </m:r>
+                      <m:r>
+                        <a:rPr lang="es-MX" sz="900" b="0" i="1">
+                          <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
+                          <a:ea typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
+                        </a:rPr>
+                        <m:t>𝑎</m:t>
+                      </m:r>
+                    </m:num>
+                    <m:den>
+                      <m:r>
+                        <a:rPr lang="es-MX" sz="900" b="0" i="1">
+                          <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
+                          <a:ea typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
+                        </a:rPr>
+                        <m:t>𝑐</m:t>
+                      </m:r>
+                      <m:r>
+                        <a:rPr lang="es-MX" sz="900" b="0" i="1">
+                          <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
+                          <a:ea typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
+                        </a:rPr>
+                        <m:t>−</m:t>
+                      </m:r>
+                      <m:r>
+                        <a:rPr lang="es-MX" sz="900" b="0" i="1">
+                          <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
+                          <a:ea typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
+                        </a:rPr>
+                        <m:t>𝑎</m:t>
+                      </m:r>
+                    </m:den>
+                  </m:f>
+                </m:oMath>
+              </a14:m>
+              <a:endParaRPr lang="es-CO" sz="900"/>
+            </a:p>
+          </xdr:txBody>
+        </xdr:sp>
+      </mc:Choice>
+      <mc:Fallback>
+        <xdr:sp macro="" textlink="">
+          <xdr:nvSpPr>
+            <xdr:cNvPr id="8" name="CuadroTexto 12">
+              <a:extLst>
+                <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{4E34FD70-1C53-4FDC-8875-98645C53E3B7}"/>
+                </a:ext>
+              </a:extLst>
+            </xdr:cNvPr>
+            <xdr:cNvSpPr txBox="1"/>
+          </xdr:nvSpPr>
+          <xdr:spPr>
+            <a:xfrm>
+              <a:off x="4080056" y="9798843"/>
+              <a:ext cx="3055793" cy="291875"/>
+            </a:xfrm>
+            <a:prstGeom prst="rect">
+              <a:avLst/>
+            </a:prstGeom>
+          </xdr:spPr>
+          <xdr:txBody>
+            <a:bodyPr vert="horz" wrap="square" lIns="91440" tIns="45720" rIns="91440" bIns="45720" rtlCol="0">
+              <a:spAutoFit/>
+            </a:bodyPr>
+            <a:lstStyle>
+              <a:defPPr>
+                <a:defRPr lang="es-CO"/>
+              </a:defPPr>
+              <a:lvl1pPr marL="0" algn="l" defTabSz="914400" rtl="0" eaLnBrk="1" latinLnBrk="0" hangingPunct="1">
+                <a:defRPr sz="1800" kern="1200">
+                  <a:solidFill>
+                    <a:schemeClr val="tx1"/>
+                  </a:solidFill>
+                  <a:latin typeface="+mn-lt"/>
+                  <a:ea typeface="+mn-ea"/>
+                  <a:cs typeface="+mn-cs"/>
+                </a:defRPr>
+              </a:lvl1pPr>
+              <a:lvl2pPr marL="457200" algn="l" defTabSz="914400" rtl="0" eaLnBrk="1" latinLnBrk="0" hangingPunct="1">
+                <a:defRPr sz="1800" kern="1200">
+                  <a:solidFill>
+                    <a:schemeClr val="tx1"/>
+                  </a:solidFill>
+                  <a:latin typeface="+mn-lt"/>
+                  <a:ea typeface="+mn-ea"/>
+                  <a:cs typeface="+mn-cs"/>
+                </a:defRPr>
+              </a:lvl2pPr>
+              <a:lvl3pPr marL="914400" algn="l" defTabSz="914400" rtl="0" eaLnBrk="1" latinLnBrk="0" hangingPunct="1">
+                <a:defRPr sz="1800" kern="1200">
+                  <a:solidFill>
+                    <a:schemeClr val="tx1"/>
+                  </a:solidFill>
+                  <a:latin typeface="+mn-lt"/>
+                  <a:ea typeface="+mn-ea"/>
+                  <a:cs typeface="+mn-cs"/>
+                </a:defRPr>
+              </a:lvl3pPr>
+              <a:lvl4pPr marL="1371600" algn="l" defTabSz="914400" rtl="0" eaLnBrk="1" latinLnBrk="0" hangingPunct="1">
+                <a:defRPr sz="1800" kern="1200">
+                  <a:solidFill>
+                    <a:schemeClr val="tx1"/>
+                  </a:solidFill>
+                  <a:latin typeface="+mn-lt"/>
+                  <a:ea typeface="+mn-ea"/>
+                  <a:cs typeface="+mn-cs"/>
+                </a:defRPr>
+              </a:lvl4pPr>
+              <a:lvl5pPr marL="1828800" algn="l" defTabSz="914400" rtl="0" eaLnBrk="1" latinLnBrk="0" hangingPunct="1">
+                <a:defRPr sz="1800" kern="1200">
+                  <a:solidFill>
+                    <a:schemeClr val="tx1"/>
+                  </a:solidFill>
+                  <a:latin typeface="+mn-lt"/>
+                  <a:ea typeface="+mn-ea"/>
+                  <a:cs typeface="+mn-cs"/>
+                </a:defRPr>
+              </a:lvl5pPr>
+              <a:lvl6pPr marL="2286000" algn="l" defTabSz="914400" rtl="0" eaLnBrk="1" latinLnBrk="0" hangingPunct="1">
+                <a:defRPr sz="1800" kern="1200">
+                  <a:solidFill>
+                    <a:schemeClr val="tx1"/>
+                  </a:solidFill>
+                  <a:latin typeface="+mn-lt"/>
+                  <a:ea typeface="+mn-ea"/>
+                  <a:cs typeface="+mn-cs"/>
+                </a:defRPr>
+              </a:lvl6pPr>
+              <a:lvl7pPr marL="2743200" algn="l" defTabSz="914400" rtl="0" eaLnBrk="1" latinLnBrk="0" hangingPunct="1">
+                <a:defRPr sz="1800" kern="1200">
+                  <a:solidFill>
+                    <a:schemeClr val="tx1"/>
+                  </a:solidFill>
+                  <a:latin typeface="+mn-lt"/>
+                  <a:ea typeface="+mn-ea"/>
+                  <a:cs typeface="+mn-cs"/>
+                </a:defRPr>
+              </a:lvl7pPr>
+              <a:lvl8pPr marL="3200400" algn="l" defTabSz="914400" rtl="0" eaLnBrk="1" latinLnBrk="0" hangingPunct="1">
+                <a:defRPr sz="1800" kern="1200">
+                  <a:solidFill>
+                    <a:schemeClr val="tx1"/>
+                  </a:solidFill>
+                  <a:latin typeface="+mn-lt"/>
+                  <a:ea typeface="+mn-ea"/>
+                  <a:cs typeface="+mn-cs"/>
+                </a:defRPr>
+              </a:lvl8pPr>
+              <a:lvl9pPr marL="3657600" algn="l" defTabSz="914400" rtl="0" eaLnBrk="1" latinLnBrk="0" hangingPunct="1">
+                <a:defRPr sz="1800" kern="1200">
+                  <a:solidFill>
+                    <a:schemeClr val="tx1"/>
+                  </a:solidFill>
+                  <a:latin typeface="+mn-lt"/>
+                  <a:ea typeface="+mn-ea"/>
+                  <a:cs typeface="+mn-cs"/>
+                </a:defRPr>
+              </a:lvl9pPr>
+            </a:lstStyle>
+            <a:p>
+              <a:r>
+                <a:rPr lang="es-MX" sz="900"/>
+                <a:t>x = a + </a:t>
+              </a:r>
+              <a:r>
+                <a:rPr lang="es-MX" sz="900" i="0">
+                  <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
+                </a:rPr>
+                <a:t>√(</a:t>
+              </a:r>
+              <a:r>
+                <a:rPr lang="es-MX" sz="900" b="0" i="0">
+                  <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
+                </a:rPr>
+                <a:t>𝑃(&lt;𝑥)(𝑏−𝑎)(𝑐−𝑎))</a:t>
+              </a:r>
+              <a:r>
+                <a:rPr lang="es-CO" sz="900"/>
+                <a:t>, 	si </a:t>
+              </a:r>
+              <a:r>
+                <a:rPr lang="es-MX" sz="900" b="0" i="0">
+                  <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
+                </a:rPr>
+                <a:t>𝑃(&lt;𝑥)≤</a:t>
+              </a:r>
+              <a:r>
+                <a:rPr lang="es-MX" sz="900" b="0" i="0">
+                  <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
+                  <a:ea typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
+                </a:rPr>
+                <a:t>(𝑏−𝑎)/(𝑐−𝑎)</a:t>
+              </a:r>
+              <a:endParaRPr lang="es-CO" sz="900"/>
+            </a:p>
+          </xdr:txBody>
+        </xdr:sp>
+      </mc:Fallback>
+    </mc:AlternateContent>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>3</xdr:col>
+      <xdr:colOff>291703</xdr:colOff>
+      <xdr:row>56</xdr:row>
+      <xdr:rowOff>137319</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>7</xdr:col>
+      <xdr:colOff>482744</xdr:colOff>
+      <xdr:row>58</xdr:row>
+      <xdr:rowOff>72007</xdr:rowOff>
+    </xdr:to>
+    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+      <mc:Choice xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" Requires="a14">
+        <xdr:sp macro="" textlink="">
+          <xdr:nvSpPr>
+            <xdr:cNvPr id="9" name="CuadroTexto 13">
+              <a:extLst>
+                <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{52FF1B47-9DC9-4A73-B72A-C3587EEDC0BC}"/>
+                </a:ext>
+              </a:extLst>
+            </xdr:cNvPr>
+            <xdr:cNvSpPr txBox="1"/>
+          </xdr:nvSpPr>
+          <xdr:spPr>
+            <a:xfrm>
+              <a:off x="4101703" y="10210007"/>
+              <a:ext cx="3697432" cy="291875"/>
+            </a:xfrm>
+            <a:prstGeom prst="rect">
+              <a:avLst/>
+            </a:prstGeom>
+          </xdr:spPr>
+          <xdr:txBody>
+            <a:bodyPr vert="horz" wrap="square" lIns="91440" tIns="45720" rIns="91440" bIns="45720" rtlCol="0">
+              <a:spAutoFit/>
+            </a:bodyPr>
+            <a:lstStyle>
+              <a:defPPr>
+                <a:defRPr lang="es-CO"/>
+              </a:defPPr>
+              <a:lvl1pPr marL="0" algn="l" defTabSz="914400" rtl="0" eaLnBrk="1" latinLnBrk="0" hangingPunct="1">
+                <a:defRPr sz="1800" kern="1200">
+                  <a:solidFill>
+                    <a:schemeClr val="tx1"/>
+                  </a:solidFill>
+                  <a:latin typeface="+mn-lt"/>
+                  <a:ea typeface="+mn-ea"/>
+                  <a:cs typeface="+mn-cs"/>
+                </a:defRPr>
+              </a:lvl1pPr>
+              <a:lvl2pPr marL="457200" algn="l" defTabSz="914400" rtl="0" eaLnBrk="1" latinLnBrk="0" hangingPunct="1">
+                <a:defRPr sz="1800" kern="1200">
+                  <a:solidFill>
+                    <a:schemeClr val="tx1"/>
+                  </a:solidFill>
+                  <a:latin typeface="+mn-lt"/>
+                  <a:ea typeface="+mn-ea"/>
+                  <a:cs typeface="+mn-cs"/>
+                </a:defRPr>
+              </a:lvl2pPr>
+              <a:lvl3pPr marL="914400" algn="l" defTabSz="914400" rtl="0" eaLnBrk="1" latinLnBrk="0" hangingPunct="1">
+                <a:defRPr sz="1800" kern="1200">
+                  <a:solidFill>
+                    <a:schemeClr val="tx1"/>
+                  </a:solidFill>
+                  <a:latin typeface="+mn-lt"/>
+                  <a:ea typeface="+mn-ea"/>
+                  <a:cs typeface="+mn-cs"/>
+                </a:defRPr>
+              </a:lvl3pPr>
+              <a:lvl4pPr marL="1371600" algn="l" defTabSz="914400" rtl="0" eaLnBrk="1" latinLnBrk="0" hangingPunct="1">
+                <a:defRPr sz="1800" kern="1200">
+                  <a:solidFill>
+                    <a:schemeClr val="tx1"/>
+                  </a:solidFill>
+                  <a:latin typeface="+mn-lt"/>
+                  <a:ea typeface="+mn-ea"/>
+                  <a:cs typeface="+mn-cs"/>
+                </a:defRPr>
+              </a:lvl4pPr>
+              <a:lvl5pPr marL="1828800" algn="l" defTabSz="914400" rtl="0" eaLnBrk="1" latinLnBrk="0" hangingPunct="1">
+                <a:defRPr sz="1800" kern="1200">
+                  <a:solidFill>
+                    <a:schemeClr val="tx1"/>
+                  </a:solidFill>
+                  <a:latin typeface="+mn-lt"/>
+                  <a:ea typeface="+mn-ea"/>
+                  <a:cs typeface="+mn-cs"/>
+                </a:defRPr>
+              </a:lvl5pPr>
+              <a:lvl6pPr marL="2286000" algn="l" defTabSz="914400" rtl="0" eaLnBrk="1" latinLnBrk="0" hangingPunct="1">
+                <a:defRPr sz="1800" kern="1200">
+                  <a:solidFill>
+                    <a:schemeClr val="tx1"/>
+                  </a:solidFill>
+                  <a:latin typeface="+mn-lt"/>
+                  <a:ea typeface="+mn-ea"/>
+                  <a:cs typeface="+mn-cs"/>
+                </a:defRPr>
+              </a:lvl6pPr>
+              <a:lvl7pPr marL="2743200" algn="l" defTabSz="914400" rtl="0" eaLnBrk="1" latinLnBrk="0" hangingPunct="1">
+                <a:defRPr sz="1800" kern="1200">
+                  <a:solidFill>
+                    <a:schemeClr val="tx1"/>
+                  </a:solidFill>
+                  <a:latin typeface="+mn-lt"/>
+                  <a:ea typeface="+mn-ea"/>
+                  <a:cs typeface="+mn-cs"/>
+                </a:defRPr>
+              </a:lvl7pPr>
+              <a:lvl8pPr marL="3200400" algn="l" defTabSz="914400" rtl="0" eaLnBrk="1" latinLnBrk="0" hangingPunct="1">
+                <a:defRPr sz="1800" kern="1200">
+                  <a:solidFill>
+                    <a:schemeClr val="tx1"/>
+                  </a:solidFill>
+                  <a:latin typeface="+mn-lt"/>
+                  <a:ea typeface="+mn-ea"/>
+                  <a:cs typeface="+mn-cs"/>
+                </a:defRPr>
+              </a:lvl8pPr>
+              <a:lvl9pPr marL="3657600" algn="l" defTabSz="914400" rtl="0" eaLnBrk="1" latinLnBrk="0" hangingPunct="1">
+                <a:defRPr sz="1800" kern="1200">
+                  <a:solidFill>
+                    <a:schemeClr val="tx1"/>
+                  </a:solidFill>
+                  <a:latin typeface="+mn-lt"/>
+                  <a:ea typeface="+mn-ea"/>
+                  <a:cs typeface="+mn-cs"/>
+                </a:defRPr>
+              </a:lvl9pPr>
+            </a:lstStyle>
+            <a:p>
+              <a:r>
+                <a:rPr lang="es-MX" sz="900"/>
+                <a:t>x = </a:t>
+              </a:r>
+              <a14:m>
+                <m:oMath xmlns:m="http://schemas.openxmlformats.org/officeDocument/2006/math">
+                  <m:r>
+                    <m:rPr>
+                      <m:sty m:val="p"/>
+                    </m:rPr>
+                    <a:rPr lang="es-MX" sz="900" b="0" i="0">
+                      <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
+                    </a:rPr>
+                    <m:t>c</m:t>
+                  </m:r>
+                  <m:r>
+                    <a:rPr lang="es-MX" sz="900" b="0" i="0">
+                      <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
+                    </a:rPr>
+                    <m:t>−</m:t>
+                  </m:r>
+                  <m:rad>
+                    <m:radPr>
+                      <m:degHide m:val="on"/>
+                      <m:ctrlPr>
+                        <a:rPr lang="es-MX" sz="900" i="1">
+                          <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
+                        </a:rPr>
+                      </m:ctrlPr>
+                    </m:radPr>
+                    <m:deg/>
+                    <m:e>
+                      <m:r>
+                        <a:rPr lang="es-MX" sz="900" b="0" i="1">
+                          <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
+                        </a:rPr>
+                        <m:t>[1−</m:t>
+                      </m:r>
+                      <m:r>
+                        <a:rPr lang="es-MX" sz="900" b="0" i="1">
+                          <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
+                        </a:rPr>
+                        <m:t>𝑃</m:t>
+                      </m:r>
+                      <m:d>
+                        <m:dPr>
+                          <m:ctrlPr>
+                            <a:rPr lang="es-MX" sz="900" b="0" i="1">
+                              <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
+                            </a:rPr>
+                          </m:ctrlPr>
+                        </m:dPr>
+                        <m:e>
+                          <m:r>
+                            <a:rPr lang="es-MX" sz="900" b="0" i="1">
+                              <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
+                            </a:rPr>
+                            <m:t>&lt;</m:t>
+                          </m:r>
+                          <m:r>
+                            <a:rPr lang="es-MX" sz="900" b="0" i="1">
+                              <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
+                            </a:rPr>
+                            <m:t>𝑥</m:t>
+                          </m:r>
+                        </m:e>
+                      </m:d>
+                      <m:r>
+                        <a:rPr lang="es-MX" sz="900" b="0" i="1">
+                          <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
+                        </a:rPr>
+                        <m:t>](</m:t>
+                      </m:r>
+                      <m:r>
+                        <a:rPr lang="es-MX" sz="900" b="0" i="1">
+                          <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
+                        </a:rPr>
+                        <m:t>𝑏</m:t>
+                      </m:r>
+                      <m:r>
+                        <a:rPr lang="es-MX" sz="900" b="0" i="1">
+                          <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
+                        </a:rPr>
+                        <m:t>−</m:t>
+                      </m:r>
+                      <m:r>
+                        <a:rPr lang="es-MX" sz="900" b="0" i="1">
+                          <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
+                        </a:rPr>
+                        <m:t>𝑎</m:t>
+                      </m:r>
+                      <m:r>
+                        <a:rPr lang="es-MX" sz="900" b="0" i="1">
+                          <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
+                        </a:rPr>
+                        <m:t>)(</m:t>
+                      </m:r>
+                      <m:r>
+                        <a:rPr lang="es-MX" sz="900" b="0" i="1">
+                          <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
+                        </a:rPr>
+                        <m:t>𝑐</m:t>
+                      </m:r>
+                      <m:r>
+                        <a:rPr lang="es-MX" sz="900" b="0" i="1">
+                          <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
+                        </a:rPr>
+                        <m:t>−</m:t>
+                      </m:r>
+                      <m:r>
+                        <a:rPr lang="es-MX" sz="900" b="0" i="1">
+                          <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
+                        </a:rPr>
+                        <m:t>𝑎</m:t>
+                      </m:r>
+                      <m:r>
+                        <a:rPr lang="es-MX" sz="900" b="0" i="1">
+                          <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
+                        </a:rPr>
+                        <m:t>)</m:t>
+                      </m:r>
+                    </m:e>
+                  </m:rad>
+                </m:oMath>
+              </a14:m>
+              <a:r>
+                <a:rPr lang="es-CO" sz="900"/>
+                <a:t>, </a:t>
+              </a:r>
+              <a:r>
+                <a:rPr lang="es-CO" sz="900" baseline="0"/>
+                <a:t>    </a:t>
+              </a:r>
+              <a:r>
+                <a:rPr lang="es-CO" sz="900"/>
+                <a:t>si </a:t>
+              </a:r>
+              <a14:m>
+                <m:oMath xmlns:m="http://schemas.openxmlformats.org/officeDocument/2006/math">
+                  <m:r>
+                    <a:rPr lang="es-MX" sz="900" b="0" i="1">
+                      <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
+                    </a:rPr>
+                    <m:t>𝑃</m:t>
+                  </m:r>
+                  <m:r>
+                    <a:rPr lang="es-MX" sz="900" b="0" i="1">
+                      <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
+                    </a:rPr>
+                    <m:t>(&lt;</m:t>
+                  </m:r>
+                  <m:r>
+                    <a:rPr lang="es-MX" sz="900" b="0" i="1">
+                      <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
+                    </a:rPr>
+                    <m:t>𝑥</m:t>
+                  </m:r>
+                  <m:r>
+                    <a:rPr lang="es-MX" sz="900" b="0" i="1">
+                      <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
+                    </a:rPr>
+                    <m:t>)&gt;</m:t>
+                  </m:r>
+                  <m:f>
+                    <m:fPr>
+                      <m:ctrlPr>
+                        <a:rPr lang="es-MX" sz="900" b="0" i="1">
+                          <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
+                          <a:ea typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
+                        </a:rPr>
+                      </m:ctrlPr>
+                    </m:fPr>
+                    <m:num>
+                      <m:r>
+                        <a:rPr lang="es-MX" sz="900" b="0" i="1">
+                          <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
+                          <a:ea typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
+                        </a:rPr>
+                        <m:t>𝑏</m:t>
+                      </m:r>
+                      <m:r>
+                        <a:rPr lang="es-MX" sz="900" b="0" i="1">
+                          <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
+                          <a:ea typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
+                        </a:rPr>
+                        <m:t>−</m:t>
+                      </m:r>
+                      <m:r>
+                        <a:rPr lang="es-MX" sz="900" b="0" i="1">
+                          <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
+                          <a:ea typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
+                        </a:rPr>
+                        <m:t>𝑎</m:t>
+                      </m:r>
+                    </m:num>
+                    <m:den>
+                      <m:r>
+                        <a:rPr lang="es-MX" sz="900" b="0" i="1">
+                          <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
+                          <a:ea typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
+                        </a:rPr>
+                        <m:t>𝑐</m:t>
+                      </m:r>
+                      <m:r>
+                        <a:rPr lang="es-MX" sz="900" b="0" i="1">
+                          <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
+                          <a:ea typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
+                        </a:rPr>
+                        <m:t>−</m:t>
+                      </m:r>
+                      <m:r>
+                        <a:rPr lang="es-MX" sz="900" b="0" i="1">
+                          <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
+                          <a:ea typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
+                        </a:rPr>
+                        <m:t>𝑎</m:t>
+                      </m:r>
+                    </m:den>
+                  </m:f>
+                </m:oMath>
+              </a14:m>
+              <a:endParaRPr lang="es-CO" sz="900"/>
+            </a:p>
+          </xdr:txBody>
+        </xdr:sp>
+      </mc:Choice>
+      <mc:Fallback>
+        <xdr:sp macro="" textlink="">
+          <xdr:nvSpPr>
+            <xdr:cNvPr id="9" name="CuadroTexto 13">
+              <a:extLst>
+                <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{52FF1B47-9DC9-4A73-B72A-C3587EEDC0BC}"/>
+                </a:ext>
+              </a:extLst>
+            </xdr:cNvPr>
+            <xdr:cNvSpPr txBox="1"/>
+          </xdr:nvSpPr>
+          <xdr:spPr>
+            <a:xfrm>
+              <a:off x="4101703" y="10210007"/>
+              <a:ext cx="3697432" cy="291875"/>
+            </a:xfrm>
+            <a:prstGeom prst="rect">
+              <a:avLst/>
+            </a:prstGeom>
+          </xdr:spPr>
+          <xdr:txBody>
+            <a:bodyPr vert="horz" wrap="square" lIns="91440" tIns="45720" rIns="91440" bIns="45720" rtlCol="0">
+              <a:spAutoFit/>
+            </a:bodyPr>
+            <a:lstStyle>
+              <a:defPPr>
+                <a:defRPr lang="es-CO"/>
+              </a:defPPr>
+              <a:lvl1pPr marL="0" algn="l" defTabSz="914400" rtl="0" eaLnBrk="1" latinLnBrk="0" hangingPunct="1">
+                <a:defRPr sz="1800" kern="1200">
+                  <a:solidFill>
+                    <a:schemeClr val="tx1"/>
+                  </a:solidFill>
+                  <a:latin typeface="+mn-lt"/>
+                  <a:ea typeface="+mn-ea"/>
+                  <a:cs typeface="+mn-cs"/>
+                </a:defRPr>
+              </a:lvl1pPr>
+              <a:lvl2pPr marL="457200" algn="l" defTabSz="914400" rtl="0" eaLnBrk="1" latinLnBrk="0" hangingPunct="1">
+                <a:defRPr sz="1800" kern="1200">
+                  <a:solidFill>
+                    <a:schemeClr val="tx1"/>
+                  </a:solidFill>
+                  <a:latin typeface="+mn-lt"/>
+                  <a:ea typeface="+mn-ea"/>
+                  <a:cs typeface="+mn-cs"/>
+                </a:defRPr>
+              </a:lvl2pPr>
+              <a:lvl3pPr marL="914400" algn="l" defTabSz="914400" rtl="0" eaLnBrk="1" latinLnBrk="0" hangingPunct="1">
+                <a:defRPr sz="1800" kern="1200">
+                  <a:solidFill>
+                    <a:schemeClr val="tx1"/>
+                  </a:solidFill>
+                  <a:latin typeface="+mn-lt"/>
+                  <a:ea typeface="+mn-ea"/>
+                  <a:cs typeface="+mn-cs"/>
+                </a:defRPr>
+              </a:lvl3pPr>
+              <a:lvl4pPr marL="1371600" algn="l" defTabSz="914400" rtl="0" eaLnBrk="1" latinLnBrk="0" hangingPunct="1">
+                <a:defRPr sz="1800" kern="1200">
+                  <a:solidFill>
+                    <a:schemeClr val="tx1"/>
+                  </a:solidFill>
+                  <a:latin typeface="+mn-lt"/>
+                  <a:ea typeface="+mn-ea"/>
+                  <a:cs typeface="+mn-cs"/>
+                </a:defRPr>
+              </a:lvl4pPr>
+              <a:lvl5pPr marL="1828800" algn="l" defTabSz="914400" rtl="0" eaLnBrk="1" latinLnBrk="0" hangingPunct="1">
+                <a:defRPr sz="1800" kern="1200">
+                  <a:solidFill>
+                    <a:schemeClr val="tx1"/>
+                  </a:solidFill>
+                  <a:latin typeface="+mn-lt"/>
+                  <a:ea typeface="+mn-ea"/>
+                  <a:cs typeface="+mn-cs"/>
+                </a:defRPr>
+              </a:lvl5pPr>
+              <a:lvl6pPr marL="2286000" algn="l" defTabSz="914400" rtl="0" eaLnBrk="1" latinLnBrk="0" hangingPunct="1">
+                <a:defRPr sz="1800" kern="1200">
+                  <a:solidFill>
+                    <a:schemeClr val="tx1"/>
+                  </a:solidFill>
+                  <a:latin typeface="+mn-lt"/>
+                  <a:ea typeface="+mn-ea"/>
+                  <a:cs typeface="+mn-cs"/>
+                </a:defRPr>
+              </a:lvl6pPr>
+              <a:lvl7pPr marL="2743200" algn="l" defTabSz="914400" rtl="0" eaLnBrk="1" latinLnBrk="0" hangingPunct="1">
+                <a:defRPr sz="1800" kern="1200">
+                  <a:solidFill>
+                    <a:schemeClr val="tx1"/>
+                  </a:solidFill>
+                  <a:latin typeface="+mn-lt"/>
+                  <a:ea typeface="+mn-ea"/>
+                  <a:cs typeface="+mn-cs"/>
+                </a:defRPr>
+              </a:lvl7pPr>
+              <a:lvl8pPr marL="3200400" algn="l" defTabSz="914400" rtl="0" eaLnBrk="1" latinLnBrk="0" hangingPunct="1">
+                <a:defRPr sz="1800" kern="1200">
+                  <a:solidFill>
+                    <a:schemeClr val="tx1"/>
+                  </a:solidFill>
+                  <a:latin typeface="+mn-lt"/>
+                  <a:ea typeface="+mn-ea"/>
+                  <a:cs typeface="+mn-cs"/>
+                </a:defRPr>
+              </a:lvl8pPr>
+              <a:lvl9pPr marL="3657600" algn="l" defTabSz="914400" rtl="0" eaLnBrk="1" latinLnBrk="0" hangingPunct="1">
+                <a:defRPr sz="1800" kern="1200">
+                  <a:solidFill>
+                    <a:schemeClr val="tx1"/>
+                  </a:solidFill>
+                  <a:latin typeface="+mn-lt"/>
+                  <a:ea typeface="+mn-ea"/>
+                  <a:cs typeface="+mn-cs"/>
+                </a:defRPr>
+              </a:lvl9pPr>
+            </a:lstStyle>
+            <a:p>
+              <a:r>
+                <a:rPr lang="es-MX" sz="900"/>
+                <a:t>x = </a:t>
+              </a:r>
+              <a:r>
+                <a:rPr lang="es-MX" sz="900" b="0" i="0">
+                  <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
+                </a:rPr>
+                <a:t>c−</a:t>
+              </a:r>
+              <a:r>
+                <a:rPr lang="es-MX" sz="900" i="0">
+                  <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
+                </a:rPr>
+                <a:t>√(</a:t>
+              </a:r>
+              <a:r>
+                <a:rPr lang="es-MX" sz="900" b="0" i="0">
+                  <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
+                </a:rPr>
+                <a:t>[1−𝑃(&lt;𝑥)](𝑏−𝑎)(𝑐−𝑎))</a:t>
+              </a:r>
+              <a:r>
+                <a:rPr lang="es-CO" sz="900"/>
+                <a:t>, </a:t>
+              </a:r>
+              <a:r>
+                <a:rPr lang="es-CO" sz="900" baseline="0"/>
+                <a:t>    </a:t>
+              </a:r>
+              <a:r>
+                <a:rPr lang="es-CO" sz="900"/>
+                <a:t>si </a:t>
+              </a:r>
+              <a:r>
+                <a:rPr lang="es-MX" sz="900" b="0" i="0">
+                  <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
+                </a:rPr>
+                <a:t>𝑃(&lt;𝑥)&gt;</a:t>
+              </a:r>
+              <a:r>
+                <a:rPr lang="es-MX" sz="900" b="0" i="0">
+                  <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
+                  <a:ea typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
+                </a:rPr>
+                <a:t>(𝑏−𝑎)/(𝑐−𝑎)</a:t>
+              </a:r>
+              <a:endParaRPr lang="es-CO" sz="900"/>
+            </a:p>
+          </xdr:txBody>
+        </xdr:sp>
+      </mc:Fallback>
+    </mc:AlternateContent>
     <xdr:clientData/>
   </xdr:twoCellAnchor>
 </xdr:wsDr>
@@ -12245,23 +12300,23 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="29" t="s">
+      <c r="A1" s="33" t="s">
         <v>80</v>
       </c>
-      <c r="B1" s="29"/>
-      <c r="C1" s="29"/>
-      <c r="D1" s="29"/>
-      <c r="E1" s="29"/>
-      <c r="F1" s="29"/>
-      <c r="G1" s="29"/>
+      <c r="B1" s="33"/>
+      <c r="C1" s="33"/>
+      <c r="D1" s="33"/>
+      <c r="E1" s="33"/>
+      <c r="F1" s="33"/>
+      <c r="G1" s="33"/>
     </row>
     <row r="2" spans="1:7" ht="15" thickTop="1" x14ac:dyDescent="0.2">
-      <c r="A2" s="28" t="s">
+      <c r="A2" s="35" t="s">
         <v>88</v>
       </c>
-      <c r="B2" s="28"/>
-      <c r="C2" s="28"/>
-      <c r="D2" s="28"/>
+      <c r="B2" s="35"/>
+      <c r="C2" s="35"/>
+      <c r="D2" s="35"/>
       <c r="E2" s="25"/>
       <c r="F2" s="25"/>
       <c r="G2" s="25"/>
@@ -12311,7 +12366,7 @@
       <c r="B7" s="3">
         <v>4000000</v>
       </c>
-      <c r="C7" s="31">
+      <c r="C7" s="28">
         <f>+NORMDIST(B7,C3,C4,0)</f>
         <v>2.2751804742259855E-7</v>
       </c>
@@ -12332,7 +12387,7 @@
       <c r="B8" s="3">
         <v>4000000</v>
       </c>
-      <c r="C8" s="32">
+      <c r="C8" s="29">
         <f>+NORMDIST(B8,C3,C4,1)</f>
         <v>0.32105490883838306</v>
       </c>
@@ -12354,7 +12409,7 @@
         <f>+C3</f>
         <v>4731496.2750000004</v>
       </c>
-      <c r="C9" s="31">
+      <c r="C9" s="28">
         <f>+NORMDIST(B9,C3,C4,0)</f>
         <v>2.5346513703088912E-7</v>
       </c>
@@ -12373,7 +12428,7 @@
         <f>+C3</f>
         <v>4731496.2750000004</v>
       </c>
-      <c r="C10" s="32">
+      <c r="C10" s="29">
         <f>+NORMDIST(B10,C3,C4,1)</f>
         <v>0.5</v>
       </c>
@@ -12391,7 +12446,7 @@
       <c r="B11" s="3">
         <v>1000000</v>
       </c>
-      <c r="C11" s="31">
+      <c r="C11" s="28">
         <f>+NORMDIST(B11,C3,C4,0)</f>
         <v>1.5255321035535096E-8</v>
       </c>
@@ -12403,7 +12458,7 @@
       <c r="B12" s="3">
         <v>1000000</v>
       </c>
-      <c r="C12" s="32">
+      <c r="C12" s="29">
         <f>+NORMDIST(B12,C3,C4,1)</f>
         <v>8.8753065388817928E-3</v>
       </c>
@@ -12415,7 +12470,7 @@
       <c r="B13" s="3">
         <v>500000</v>
       </c>
-      <c r="C13" s="31">
+      <c r="C13" s="28">
         <f>+NORMDIST(B13,C3,C4,0)</f>
         <v>6.8301171561241813E-9</v>
       </c>
@@ -12427,7 +12482,7 @@
       <c r="B14" s="3">
         <v>500000</v>
       </c>
-      <c r="C14" s="32">
+      <c r="C14" s="29">
         <f>+NORMDIST(B14,C3,C4,1)</f>
         <v>3.5892182305537704E-3</v>
       </c>
@@ -12439,7 +12494,7 @@
       <c r="B15" s="3">
         <v>-100000</v>
       </c>
-      <c r="C15" s="33">
+      <c r="C15" s="30">
         <f>+NORMDIST(B15,C3,C4,0)</f>
         <v>2.279212512429407E-9</v>
       </c>
@@ -12451,7 +12506,7 @@
       <c r="B16" s="3">
         <v>-100000</v>
       </c>
-      <c r="C16" s="32">
+      <c r="C16" s="29">
         <f>+NORMDIST(B16,C3,C4,1)</f>
         <v>1.0715245586945105E-3</v>
       </c>
@@ -12472,7 +12527,7 @@
       <c r="A19" s="24">
         <v>9.9999999999999995E-7</v>
       </c>
-      <c r="B19" s="34">
+      <c r="B19" s="31">
         <f>+NORMINV(A19,C3,C4)</f>
         <v>-2750171.4434535606</v>
       </c>
@@ -12484,27 +12539,27 @@
       <c r="A20" s="22">
         <v>0.1</v>
       </c>
-      <c r="B20" s="34">
+      <c r="B20" s="31">
         <f>+NORMINV(A20,C3,C4)</f>
         <v>2714394.0020823544</v>
       </c>
-      <c r="C20" s="30"/>
+      <c r="C20" s="27"/>
     </row>
     <row r="21" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A21" s="22">
         <v>0.32</v>
       </c>
-      <c r="B21" s="34">
+      <c r="B21" s="31">
         <f>+NORMINV(A21,C3,C4)</f>
         <v>3995360.2223443054</v>
       </c>
-      <c r="C21" s="30"/>
+      <c r="C21" s="27"/>
     </row>
     <row r="22" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A22" s="22">
         <v>0.4</v>
       </c>
-      <c r="B22" s="34">
+      <c r="B22" s="31">
         <f>+NORMINV(A22,C3,C4)</f>
         <v>4332739.7744333139</v>
       </c>
@@ -12514,7 +12569,7 @@
       <c r="A23" s="22">
         <v>0.5</v>
       </c>
-      <c r="B23" s="34">
+      <c r="B23" s="31">
         <f>+NORMINV(A23,C3,C4)</f>
         <v>4731496.2750000004</v>
       </c>
@@ -12524,7 +12579,7 @@
       <c r="A24" s="22">
         <v>0.7</v>
       </c>
-      <c r="B24" s="34">
+      <c r="B24" s="31">
         <f>+NORMINV(A24,C3,C4)</f>
         <v>5556878.1749886014</v>
       </c>
@@ -12534,7 +12589,7 @@
       <c r="A25" s="23">
         <v>0.99999000000000005</v>
       </c>
-      <c r="B25" s="34">
+      <c r="B25" s="31">
         <f>+NORMINV(A25,C3,C4)</f>
         <v>11444235.071829889</v>
       </c>
@@ -12545,15 +12600,15 @@
       <c r="C26" s="19"/>
     </row>
     <row r="28" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A28" s="29" t="s">
+      <c r="A28" s="33" t="s">
         <v>81</v>
       </c>
-      <c r="B28" s="29"/>
-      <c r="C28" s="29"/>
-      <c r="D28" s="29"/>
-      <c r="E28" s="29"/>
-      <c r="F28" s="29"/>
-      <c r="G28" s="29"/>
+      <c r="B28" s="33"/>
+      <c r="C28" s="33"/>
+      <c r="D28" s="33"/>
+      <c r="E28" s="33"/>
+      <c r="F28" s="33"/>
+      <c r="G28" s="33"/>
     </row>
     <row r="29" spans="1:7" ht="15" thickTop="1" x14ac:dyDescent="0.2">
       <c r="B29" s="1" t="s">
@@ -12577,7 +12632,7 @@
         <f>+(B30-C3)/C4</f>
         <v>-0.46475094942028661</v>
       </c>
-      <c r="D30" s="32">
+      <c r="D30" s="29">
         <f>+_xlfn.NORM.S.DIST(C30,1)</f>
         <v>0.32105490883838306</v>
       </c>
@@ -12606,11 +12661,11 @@
       <c r="A33" s="24">
         <v>9.9999999999999995E-7</v>
       </c>
-      <c r="B33" s="35">
+      <c r="B33" s="32">
         <f>+_xlfn.NORM.S.INV(A33)</f>
         <v>-4.7534243088228987</v>
       </c>
-      <c r="C33" s="34">
+      <c r="C33" s="31">
         <f>B33*C4+C3</f>
         <v>-2750171.4434535606</v>
       </c>
@@ -12619,11 +12674,11 @@
       <c r="A34" s="22">
         <v>0.1</v>
       </c>
-      <c r="B34" s="35">
+      <c r="B34" s="32">
         <f t="shared" ref="B34:B39" si="0">+_xlfn.NORM.S.INV(A34)</f>
         <v>-1.2815515655446006</v>
       </c>
-      <c r="C34" s="34">
+      <c r="C34" s="31">
         <f>B34*$C$4+$C$3</f>
         <v>2714394.0020823544</v>
       </c>
@@ -12632,11 +12687,11 @@
       <c r="A35" s="22">
         <v>0.32</v>
       </c>
-      <c r="B35" s="35">
+      <c r="B35" s="32">
         <f t="shared" si="0"/>
         <v>-0.46769879911450829</v>
       </c>
-      <c r="C35" s="34">
+      <c r="C35" s="31">
         <f t="shared" ref="C35:C39" si="1">B35*$C$4+$C$3</f>
         <v>3995360.2223443054</v>
       </c>
@@ -12645,11 +12700,11 @@
       <c r="A36" s="22">
         <v>0.4</v>
       </c>
-      <c r="B36" s="35">
+      <c r="B36" s="32">
         <f t="shared" si="0"/>
         <v>-0.25334710313579978</v>
       </c>
-      <c r="C36" s="34">
+      <c r="C36" s="31">
         <f t="shared" si="1"/>
         <v>4332739.7744333139</v>
       </c>
@@ -12658,11 +12713,11 @@
       <c r="A37" s="22">
         <v>0.5</v>
       </c>
-      <c r="B37" s="35">
+      <c r="B37" s="32">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="C37" s="34">
+      <c r="C37" s="31">
         <f t="shared" si="1"/>
         <v>4731496.2750000004</v>
       </c>
@@ -12671,11 +12726,11 @@
       <c r="A38" s="22">
         <v>0.7</v>
       </c>
-      <c r="B38" s="35">
+      <c r="B38" s="32">
         <f t="shared" si="0"/>
         <v>0.52440051270804078</v>
       </c>
-      <c r="C38" s="34">
+      <c r="C38" s="31">
         <f t="shared" si="1"/>
         <v>5556878.1749886014</v>
       </c>
@@ -12684,33 +12739,33 @@
       <c r="A39" s="23">
         <v>0.99999000000000005</v>
       </c>
-      <c r="B39" s="35">
+      <c r="B39" s="32">
         <f t="shared" si="0"/>
         <v>4.2648907939238399</v>
       </c>
-      <c r="C39" s="34">
+      <c r="C39" s="31">
         <f t="shared" si="1"/>
         <v>11444235.071829889</v>
       </c>
     </row>
     <row r="42" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A42" s="29" t="s">
+      <c r="A42" s="33" t="s">
         <v>87</v>
       </c>
-      <c r="B42" s="29"/>
-      <c r="C42" s="29"/>
-      <c r="D42" s="29"/>
-      <c r="E42" s="29"/>
-      <c r="F42" s="29"/>
-      <c r="G42" s="29"/>
+      <c r="B42" s="33"/>
+      <c r="C42" s="33"/>
+      <c r="D42" s="33"/>
+      <c r="E42" s="33"/>
+      <c r="F42" s="33"/>
+      <c r="G42" s="33"/>
     </row>
     <row r="43" spans="1:7" ht="15" thickTop="1" x14ac:dyDescent="0.2">
-      <c r="A43" s="27" t="s">
+      <c r="A43" s="34" t="s">
         <v>88</v>
       </c>
-      <c r="B43" s="27"/>
-      <c r="C43" s="27"/>
-      <c r="D43" s="27"/>
+      <c r="B43" s="34"/>
+      <c r="C43" s="34"/>
+      <c r="D43" s="34"/>
     </row>
     <row r="44" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A44" s="2" t="s">
@@ -12772,7 +12827,7 @@
       <c r="B49" s="3">
         <v>4000000</v>
       </c>
-      <c r="C49" s="31">
+      <c r="C49" s="28">
         <f>+IF(B49&lt;=C45,2*(B49-C44)/((C45-C44)*(C46-C44)),2*(C46-B49)/((C46-C45)*(C46-C44)))</f>
         <v>1.8115943934589707E-7</v>
       </c>
@@ -12793,7 +12848,7 @@
       <c r="B50" s="3">
         <v>4000000</v>
       </c>
-      <c r="C50" s="32">
+      <c r="C50" s="29">
         <f>+IF(B50&lt;=C45,(B50-C44)^2/((C45-C44)*(C46-C44)),1-(C46-B50)^2/((C46-C45)*(C46-C44)))</f>
         <v>0.28079713098614045</v>
       </c>
@@ -12819,86 +12874,86 @@
       <c r="A53" s="24">
         <v>9.9999999999999995E-7</v>
       </c>
-      <c r="B53" s="34">
-        <f>+IF(A53&lt;=(C45-C44)/(C46-C44),C44+SQRT(A53*C45*(C46-C44)),C46+SQRT((1-A53)*(C45-C44)*(C46-C44)))</f>
-        <v>906337.50711242203</v>
+      <c r="B53" s="31">
+        <f>+IF(A53&lt;=(C45-C44)/(C46-C44),C44+SQRT(A53*(C45-C44)*(C46-C44)),C46-SQRT((1-A53)*(C45-C44)*(C46-C44)))</f>
+        <v>905850.12789603788</v>
       </c>
       <c r="C53" s="2" t="s">
-        <v>116</v>
+        <v>122</v>
       </c>
     </row>
     <row r="54" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A54" s="22">
         <v>0.1</v>
       </c>
-      <c r="B54" s="34">
-        <f>+IF(A54&lt;=($C$45-$C$44)/($C$46-$C$44),$C$44+SQRT(A54*$C$45*($C$46-$C$44)),$C$46+SQRT((1-A54)*($C$45-$C$44)*($C$46-$C$44)))</f>
-        <v>2904095.7162770443</v>
+      <c r="B54" s="31">
+        <f>+IF(A54&lt;=($C$45-$C$44)/($C$46-$C$44),$C$44+SQRT(A54*($C$45-$C$44)*($C$46-$C$44)),$C$46-SQRT((1-A54)*($C$45-$C$44)*($C$46-$C$44)))</f>
+        <v>2749972.8754768269</v>
       </c>
     </row>
     <row r="55" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A55" s="22">
         <v>0.32</v>
       </c>
-      <c r="B55" s="34">
-        <f t="shared" ref="B55:B59" si="2">+IF(A55&lt;=($C$45-$C$44)/($C$46-$C$44),$C$44+SQRT(A55*$C$45*($C$46-$C$44)),$C$46+SQRT((1-A55)*($C$45-$C$44)*($C$46-$C$44)))</f>
-        <v>4485035.4040092826</v>
+      <c r="B55" s="31">
+        <f t="shared" ref="B55:B59" si="2">+IF(A55&lt;=($C$45-$C$44)/($C$46-$C$44),$C$44+SQRT(A55*($C$45-$C$44)*($C$46-$C$44)),$C$46-SQRT((1-A55)*($C$45-$C$44)*($C$46-$C$44)))</f>
+        <v>4209332.0848775506</v>
       </c>
     </row>
     <row r="56" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A56" s="22">
         <v>0.4</v>
       </c>
-      <c r="B56" s="34">
+      <c r="B56" s="31">
         <f t="shared" si="2"/>
-        <v>4908191.4325540885</v>
+        <v>4599945.7509536538</v>
       </c>
     </row>
     <row r="57" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A57" s="22">
         <v>0.5</v>
       </c>
-      <c r="B57" s="34">
+      <c r="B57" s="31">
         <f t="shared" si="2"/>
-        <v>5381294.2550116032</v>
+        <v>5036665.1060969392</v>
       </c>
     </row>
     <row r="58" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A58" s="22">
         <v>0.7</v>
       </c>
-      <c r="B58" s="34">
+      <c r="B58" s="31">
         <f t="shared" si="2"/>
-        <v>6202338.8688389203</v>
+        <v>5794568.1607267456</v>
       </c>
     </row>
     <row r="59" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A59" s="23">
         <v>0.99999000000000005</v>
       </c>
-      <c r="B59" s="34">
+      <c r="B59" s="31">
         <f t="shared" si="2"/>
-        <v>7518499.7287547262</v>
+        <v>7481500.2712452738</v>
       </c>
     </row>
     <row r="61" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A61" s="29" t="s">
+      <c r="A61" s="33" t="s">
         <v>93</v>
       </c>
-      <c r="B61" s="29"/>
-      <c r="C61" s="29"/>
-      <c r="D61" s="29"/>
-      <c r="E61" s="29"/>
-      <c r="F61" s="29"/>
-      <c r="G61" s="29"/>
+      <c r="B61" s="33"/>
+      <c r="C61" s="33"/>
+      <c r="D61" s="33"/>
+      <c r="E61" s="33"/>
+      <c r="F61" s="33"/>
+      <c r="G61" s="33"/>
     </row>
     <row r="62" spans="1:7" ht="15" thickTop="1" x14ac:dyDescent="0.2">
-      <c r="A62" s="27" t="s">
+      <c r="A62" s="34" t="s">
         <v>88</v>
       </c>
-      <c r="B62" s="27"/>
-      <c r="C62" s="27"/>
-      <c r="D62" s="27"/>
+      <c r="B62" s="34"/>
+      <c r="C62" s="34"/>
+      <c r="D62" s="34"/>
     </row>
     <row r="63" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A63" s="2" t="s">
@@ -12939,7 +12994,7 @@
       <c r="B67" s="3">
         <v>4000000</v>
       </c>
-      <c r="C67" s="31">
+      <c r="C67" s="28">
         <f>1/(B64-B63)</f>
         <v>1.5151515151515152E-7</v>
       </c>
@@ -12950,7 +13005,7 @@
         <v>78</v>
       </c>
       <c r="F67" s="2" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
     </row>
     <row r="68" spans="1:7" x14ac:dyDescent="0.2">
@@ -12960,7 +13015,7 @@
       <c r="B68" s="3">
         <v>4000000</v>
       </c>
-      <c r="C68" s="32">
+      <c r="C68" s="29">
         <f>+(B68-B63)/(B64-B63)</f>
         <v>0.46969696969696972</v>
       </c>
@@ -12971,7 +13026,7 @@
         <v>79</v>
       </c>
       <c r="F68" s="2" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
     </row>
     <row r="70" spans="1:7" x14ac:dyDescent="0.2">
@@ -12986,19 +13041,19 @@
       <c r="A71" s="24">
         <v>9.9999999999999995E-7</v>
       </c>
-      <c r="B71" s="34">
+      <c r="B71" s="31">
         <f>+B63+A71*(B64-B63)</f>
         <v>900006.6</v>
       </c>
       <c r="C71" s="2" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
     </row>
     <row r="72" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A72" s="22">
         <v>0.1</v>
       </c>
-      <c r="B72" s="34">
+      <c r="B72" s="31">
         <f>+$B$63+A72*($B$64-$B$63)</f>
         <v>1560000</v>
       </c>
@@ -13007,7 +13062,7 @@
       <c r="A73" s="22">
         <v>0.32</v>
       </c>
-      <c r="B73" s="34">
+      <c r="B73" s="31">
         <f t="shared" ref="B73:B77" si="3">+$B$63+A73*($B$64-$B$63)</f>
         <v>3012000</v>
       </c>
@@ -13016,7 +13071,7 @@
       <c r="A74" s="22">
         <v>0.4</v>
       </c>
-      <c r="B74" s="34">
+      <c r="B74" s="31">
         <f t="shared" si="3"/>
         <v>3540000</v>
       </c>
@@ -13025,7 +13080,7 @@
       <c r="A75" s="22">
         <v>0.5</v>
       </c>
-      <c r="B75" s="34">
+      <c r="B75" s="31">
         <f t="shared" si="3"/>
         <v>4200000</v>
       </c>
@@ -13034,7 +13089,7 @@
       <c r="A76" s="22">
         <v>0.7</v>
       </c>
-      <c r="B76" s="34">
+      <c r="B76" s="31">
         <f t="shared" si="3"/>
         <v>5520000</v>
       </c>
@@ -13043,29 +13098,29 @@
       <c r="A77" s="23">
         <v>0.99999000000000005</v>
       </c>
-      <c r="B77" s="34">
+      <c r="B77" s="31">
         <f t="shared" si="3"/>
         <v>7499934</v>
       </c>
     </row>
     <row r="80" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A80" s="29" t="s">
+      <c r="A80" s="33" t="s">
         <v>97</v>
       </c>
-      <c r="B80" s="29"/>
-      <c r="C80" s="29"/>
-      <c r="D80" s="29"/>
-      <c r="E80" s="29"/>
-      <c r="F80" s="29"/>
-      <c r="G80" s="29"/>
+      <c r="B80" s="33"/>
+      <c r="C80" s="33"/>
+      <c r="D80" s="33"/>
+      <c r="E80" s="33"/>
+      <c r="F80" s="33"/>
+      <c r="G80" s="33"/>
     </row>
     <row r="81" spans="1:6" ht="15" thickTop="1" x14ac:dyDescent="0.2">
-      <c r="A81" s="28" t="s">
+      <c r="A81" s="35" t="s">
         <v>88</v>
       </c>
-      <c r="B81" s="28"/>
-      <c r="C81" s="28"/>
-      <c r="D81" s="28"/>
+      <c r="B81" s="35"/>
+      <c r="C81" s="35"/>
+      <c r="D81" s="35"/>
     </row>
     <row r="82" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A82" s="2" t="s">
@@ -13112,7 +13167,7 @@
       <c r="B86" s="3">
         <v>4000000</v>
       </c>
-      <c r="C86" s="33">
+      <c r="C86" s="30">
         <f>+_xlfn.LOGNORM.DIST(B86,C82,C83,0)</f>
         <v>2.0876386597122864E-7</v>
       </c>
@@ -13123,7 +13178,7 @@
         <v>78</v>
       </c>
       <c r="F86" s="2" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
     </row>
     <row r="87" spans="1:6" x14ac:dyDescent="0.2">
@@ -13133,7 +13188,7 @@
       <c r="B87" s="3">
         <v>4000000</v>
       </c>
-      <c r="C87" s="32">
+      <c r="C87" s="29">
         <f>+_xlfn.LOGNORM.DIST(B87,C82,C83,1)</f>
         <v>0.4290668557854399</v>
       </c>
@@ -13144,7 +13199,7 @@
         <v>79</v>
       </c>
       <c r="F87" s="2" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
     </row>
     <row r="88" spans="1:6" x14ac:dyDescent="0.2">
@@ -13155,7 +13210,7 @@
         <f>+C3</f>
         <v>4731496.2750000004</v>
       </c>
-      <c r="C88" s="33">
+      <c r="C88" s="30">
         <f>+_xlfn.LOGNORM.DIST(B88,C82,C83,0)</f>
         <v>1.7649802637250393E-7</v>
       </c>
@@ -13174,7 +13229,7 @@
         <f>+B88</f>
         <v>4731496.2750000004</v>
       </c>
-      <c r="C89" s="32">
+      <c r="C89" s="29">
         <f>+_xlfn.LOGNORM.DIST(B89,C82,C83,1)</f>
         <v>0.57081654906962087</v>
       </c>
@@ -13192,7 +13247,7 @@
       <c r="B90" s="3">
         <v>1000000</v>
       </c>
-      <c r="C90" s="33">
+      <c r="C90" s="30">
         <f>+_xlfn.LOGNORM.DIST(B90,C82,C83,0)</f>
         <v>6.3832231671053696E-9</v>
       </c>
@@ -13204,7 +13259,7 @@
       <c r="B91" s="3">
         <v>1000000</v>
       </c>
-      <c r="C91" s="32">
+      <c r="C91" s="29">
         <f>+_xlfn.LOGNORM.DIST(B91,C82,C83,1)</f>
         <v>8.822926966381724E-4</v>
       </c>
@@ -13216,7 +13271,7 @@
       <c r="B92" s="3">
         <v>8000000</v>
       </c>
-      <c r="C92" s="33">
+      <c r="C92" s="30">
         <f>+_xlfn.LOGNORM.DIST(B92,C82,C83,0)</f>
         <v>4.5827414164616569E-8</v>
       </c>
@@ -13229,7 +13284,7 @@
         <f>+B92</f>
         <v>8000000</v>
       </c>
-      <c r="C93" s="32">
+      <c r="C93" s="29">
         <f>+_xlfn.LOGNORM.DIST(B93,C82,C83,1)</f>
         <v>0.90242474929620942</v>
       </c>
@@ -13241,7 +13296,7 @@
       <c r="B94" s="3">
         <v>-100000</v>
       </c>
-      <c r="C94" s="33" t="e">
+      <c r="C94" s="30" t="e">
         <f>+_xlfn.LOGNORM.DIST(B94,C82,C83,0)</f>
         <v>#NUM!</v>
       </c>
@@ -13253,7 +13308,7 @@
       <c r="B95" s="3">
         <v>-100000</v>
       </c>
-      <c r="C95" s="33" t="e">
+      <c r="C95" s="30" t="e">
         <f>+_xlfn.LOGNORM.DIST(B95,C82,C83,1)</f>
         <v>#NUM!</v>
       </c>
@@ -13270,19 +13325,19 @@
       <c r="A98" s="24">
         <v>9.9999999999999995E-7</v>
       </c>
-      <c r="B98" s="34">
+      <c r="B98" s="31">
         <f>+LOGINV(A98,C82,C83)</f>
         <v>465525.6710889184</v>
       </c>
       <c r="C98" s="2" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
     </row>
     <row r="99" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A99" s="22">
         <v>0.1</v>
       </c>
-      <c r="B99" s="34">
+      <c r="B99" s="31">
         <f>+LOGINV(A99,$C$82,$C$83)</f>
         <v>2381637.8144874666</v>
       </c>
@@ -13291,7 +13346,7 @@
       <c r="A100" s="22">
         <v>0.32</v>
       </c>
-      <c r="B100" s="34">
+      <c r="B100" s="31">
         <f t="shared" ref="B100:B104" si="4">+LOGINV(A100,$C$82,$C$83)</f>
         <v>3491875.4801146644</v>
       </c>
@@ -13300,7 +13355,7 @@
       <c r="A101" s="22">
         <v>0.4</v>
       </c>
-      <c r="B101" s="34">
+      <c r="B101" s="31">
         <f t="shared" si="4"/>
         <v>3862138.6650704285</v>
       </c>
@@ -13309,7 +13364,7 @@
       <c r="A102" s="22">
         <v>0.5</v>
       </c>
-      <c r="B102" s="34">
+      <c r="B102" s="31">
         <f t="shared" si="4"/>
         <v>4350704.2840180723</v>
       </c>
@@ -13318,7 +13373,7 @@
       <c r="A103" s="22">
         <v>0.7</v>
       </c>
-      <c r="B103" s="34">
+      <c r="B103" s="31">
         <f t="shared" si="4"/>
         <v>5567221.1706368346</v>
       </c>
@@ -13327,7 +13382,7 @@
       <c r="A104" s="23">
         <v>0.99999000000000005</v>
       </c>
-      <c r="B104" s="34">
+      <c r="B104" s="31">
         <f t="shared" si="4"/>
         <v>32316206.608740821</v>
       </c>

</xml_diff>